<commit_message>
📊 Horarios actualizados Línea 141 - 4631
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:15:31</t>
+          <t>Última actualización: 01:01:21</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>00:15:31</t>
+          <t>01:01:21</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>70</v>
+        <v>24</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -519,7 +519,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:15:31</t>
+          <t>Última actualización: 01:01:21</t>
         </is>
       </c>
     </row>
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:15:31</t>
+          <t>Última actualización: 01:01:21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4632
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:01:21</t>
+          <t>Última actualización: 01:47:15</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>01:01:21</t>
+          <t>01:47:15</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01:25</t>
+          <t>03:02</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>24</v>
+        <v>75</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -519,7 +519,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:01:21</t>
+          <t>Última actualización: 01:47:15</t>
         </is>
       </c>
     </row>
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:01:21</t>
+          <t>Última actualización: 01:47:15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4633
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:47:15</t>
+          <t>Última actualización: 02:13:50</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -473,12 +473,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>01:47:15</t>
+          <t>02:13:50</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:02</t>
+          <t>03:01</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -487,9 +487,59 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>75</v>
+        <v>48</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>02:13:50</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>03:48</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>95</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>02:13:50</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>04:01</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>108</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -519,7 +569,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:47:15</t>
+          <t>Última actualización: 02:13:50</t>
         </is>
       </c>
     </row>
@@ -554,7 +604,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:47:15</t>
+          <t>Última actualización: 02:13:50</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4634
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:13:50</t>
+          <t>Última actualización: 02:45:26</t>
         </is>
       </c>
     </row>
@@ -473,12 +473,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:13:50</t>
+          <t>02:45:26</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:01</t>
+          <t>03:02</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>48</v>
+        <v>17</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,7 +498,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>02:13:50</t>
+          <t>02:45:26</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>95</v>
+        <v>63</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,12 +523,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>02:13:50</t>
+          <t>02:45:26</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:01</t>
+          <t>04:02</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>108</v>
+        <v>77</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:13:50</t>
+          <t>Última actualización: 02:45:26</t>
         </is>
       </c>
     </row>
@@ -604,7 +604,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:13:50</t>
+          <t>Última actualización: 02:45:26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4635
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:45:26</t>
+          <t>Última actualización: 03:02:22</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:45:26</t>
+          <t>03:02:22</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,7 +498,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>02:45:26</t>
+          <t>03:02:22</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,7 +523,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>02:45:26</t>
+          <t>03:02:22</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -537,9 +537,59 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>03:02:22</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>04:48</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>106</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>03:02:22</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>04:53</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>111</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -569,7 +619,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:45:26</t>
+          <t>Última actualización: 03:02:22</t>
         </is>
       </c>
     </row>
@@ -604,7 +654,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:45:26</t>
+          <t>Última actualización: 03:02:22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4636
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:02:22</t>
+          <t>Última actualización: 03:55:18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>03:02:22</t>
+          <t>03:55:18</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:02</t>
+          <t>03:56</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>03:02:22</t>
+          <t>03:55:18</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>04:02</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>46</v>
+        <v>7</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,12 +523,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>03:02:22</t>
+          <t>03:55:18</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:02</t>
+          <t>04:48</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>03:02:22</t>
+          <t>03:55:18</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>04:48</t>
+          <t>04:53</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>106</v>
+        <v>58</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,23 +573,98 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>03:02:22</t>
+          <t>03:55:18</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>04:53</t>
+          <t>05:17</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>111</v>
+        <v>82</v>
       </c>
       <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>03:55:18</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>05:22</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>87</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>03:55:18</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>05:47</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>112</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>03:55:18</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>05:52</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>117</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -619,7 +694,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:02:22</t>
+          <t>Última actualización: 03:55:18</t>
         </is>
       </c>
     </row>
@@ -654,7 +729,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:02:22</t>
+          <t>Última actualización: 03:55:18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4637
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:55:18</t>
+          <t>Última actualización: 04:23:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 9</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>03:55:18</t>
+          <t>04:23:40</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:56</t>
+          <t>04:47</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>03:55:18</t>
+          <t>04:23:40</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>04:02</t>
+          <t>04:53</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>03:55:18</t>
+          <t>04:23:40</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:48</t>
+          <t>05:17</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>03:55:18</t>
+          <t>04:23:40</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>04:53</t>
+          <t>05:22</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>03:55:18</t>
+          <t>04:23:40</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05:17</t>
+          <t>05:47</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>03:55:18</t>
+          <t>04:23:40</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>05:49</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>03:55:18</t>
+          <t>04:23:40</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>05:47</t>
+          <t>06:01</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>112</v>
+        <v>98</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,23 +648,48 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>03:55:18</t>
+          <t>04:23:40</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>05:52</t>
+          <t>06:09</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>04:23:40</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>109</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -681,7 +706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -694,14 +719,66 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:55:18</t>
+          <t>Última actualización: 04:23:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>04:23:40</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>109</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
         </is>
       </c>
     </row>
@@ -729,7 +806,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:55:18</t>
+          <t>Última actualización: 04:23:40</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4638
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:23:40</t>
+          <t>Última actualización: 04:53:09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 9</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:23:40</t>
+          <t>04:53:09</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>04:47</t>
+          <t>04:53</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04:23:40</t>
+          <t>04:53:09</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>04:53</t>
+          <t>05:17</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04:23:40</t>
+          <t>04:53:09</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05:17</t>
+          <t>05:22</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04:23:40</t>
+          <t>04:53:09</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>05:44</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,7 +573,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:23:40</t>
+          <t>04:53:09</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>84</v>
+        <v>54</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:23:40</t>
+          <t>04:53:09</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05:49</t>
+          <t>06:01</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>04:23:40</t>
+          <t>04:53:09</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:01</t>
+          <t>06:09</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>98</v>
+        <v>76</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>04:23:40</t>
+          <t>04:53:09</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:09</t>
+          <t>06:12</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>106</v>
+        <v>79</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,23 +673,123 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>04:23:40</t>
+          <t>04:53:09</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>04:53:09</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>06:36</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>103</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>04:53:09</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>06:39</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>106</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>04:53:09</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>108</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>04:53:09</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>108</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -719,7 +819,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:23:40</t>
+          <t>Última actualización: 04:53:09</t>
         </is>
       </c>
     </row>
@@ -760,7 +860,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:23:40</t>
+          <t>04:53:09</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -774,7 +874,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>109</v>
+        <v>79</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -806,7 +906,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:23:40</t>
+          <t>Última actualización: 04:53:09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4639
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:53:09</t>
+          <t>Última actualización: 05:15:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:53:09</t>
+          <t>05:15:37</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>04:53</t>
+          <t>05:17</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04:53:09</t>
+          <t>05:15:37</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>05:17</t>
+          <t>05:22</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,17 +523,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04:53:09</t>
+          <t>05:15:37</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>05:44</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04:53:09</t>
+          <t>05:15:37</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05:44</t>
+          <t>05:47</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:53:09</t>
+          <t>05:15:37</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05:47</t>
+          <t>06:01</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:53:09</t>
+          <t>05:15:37</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06:01</t>
+          <t>06:09</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>04:53:09</t>
+          <t>05:15:37</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:09</t>
+          <t>06:12</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>76</v>
+        <v>57</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>04:53:09</t>
+          <t>05:15:37</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>04:53:09</t>
+          <t>05:15:37</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:36</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>04:53:09</t>
+          <t>05:15:37</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06:36</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>103</v>
+        <v>84</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>04:53:09</t>
+          <t>05:15:37</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>106</v>
+        <v>86</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>04:53:09</t>
+          <t>05:15:37</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>108</v>
+        <v>86</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,23 +773,48 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>04:53:09</t>
+          <t>05:15:37</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>05:15:37</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>07:02</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>107</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -806,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -819,14 +844,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:53:09</t>
+          <t>Última actualización: 05:15:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 2</t>
         </is>
       </c>
     </row>
@@ -860,7 +885,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:53:09</t>
+          <t>05:15:37</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -874,9 +899,34 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>79</v>
+        <v>57</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>05:15:37</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>07:02</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>107</v>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -906,7 +956,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:53:09</t>
+          <t>Última actualización: 05:15:37</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4640
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:15:37</t>
+          <t>Última actualización: 05:48:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:15:37</t>
+          <t>05:48:48</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>05:17</t>
+          <t>05:48</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:15:37</t>
+          <t>05:48:48</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>06:09</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:15:37</t>
+          <t>05:48:48</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05:44</t>
+          <t>06:12</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>05:15:37</t>
+          <t>05:48:48</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05:47</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05:15:37</t>
+          <t>05:48:48</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06:01</t>
+          <t>06:36</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>05:15:37</t>
+          <t>05:48:48</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06:09</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05:15:37</t>
+          <t>05:48:48</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>06:40</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:15:37</t>
+          <t>05:48:48</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>75</v>
+        <v>53</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>05:15:37</t>
+          <t>05:48:48</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:36</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>05:15:37</t>
+          <t>05:48:48</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>07:02</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:15:37</t>
+          <t>05:48:48</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>05:15:37</t>
+          <t>05:48:48</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>86</v>
+        <v>99</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>05:15:37</t>
+          <t>05:48:48</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>06:59</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,23 +798,73 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>05:15:37</t>
+          <t>05:48:48</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>07:02</t>
+          <t>07:31</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>05:48:48</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>108</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>05:48:48</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>07:44</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>116</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -831,7 +881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -844,14 +894,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:15:37</t>
+          <t>Última actualización: 05:48:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -885,7 +935,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:15:37</t>
+          <t>05:48:48</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -899,7 +949,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -910,7 +960,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:15:37</t>
+          <t>05:48:48</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -924,9 +974,34 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>107</v>
+        <v>74</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>05:48:48</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>07:31</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>103</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -956,7 +1031,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:15:37</t>
+          <t>Última actualización: 05:48:48</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4641
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:48:48</t>
+          <t>Última actualización: 06:11:46</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:48:48</t>
+          <t>06:11:46</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>05:48</t>
+          <t>06:12</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,12 +498,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:48:48</t>
+          <t>06:11:46</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>06:09</t>
+          <t>06:13</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:48:48</t>
+          <t>06:11:46</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>05:48:48</t>
+          <t>06:11:46</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:36</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05:48:48</t>
+          <t>06:11:46</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06:36</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>05:48:48</t>
+          <t>06:11:46</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>06:40</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05:48:48</t>
+          <t>06:11:46</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:40</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:48:48</t>
+          <t>06:11:46</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>05:48:48</t>
+          <t>06:11:46</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:59</t>
+          <t>07:02</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>71</v>
+        <v>51</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>05:48:48</t>
+          <t>06:11:46</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>07:02</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:48:48</t>
+          <t>06:11:46</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>07:20</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>92</v>
+        <v>75</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>05:48:48</t>
+          <t>06:11:46</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -762,7 +762,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>99</v>
+        <v>76</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>05:48:48</t>
+          <t>06:11:46</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>07:27</t>
+          <t>07:31</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,21 +798,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>05:48:48</t>
+          <t>06:11:46</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>07:31</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,21 +823,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>05:48:48</t>
+          <t>06:11:46</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:44</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>108</v>
+        <v>93</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,21 +848,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>05:48:48</t>
+          <t>06:11:46</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>07:44</t>
+          <t>08:06</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -894,7 +894,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:48:48</t>
+          <t>Última actualización: 06:11:46</t>
         </is>
       </c>
     </row>
@@ -935,7 +935,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:48:48</t>
+          <t>06:11:46</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -960,7 +960,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:48:48</t>
+          <t>06:11:46</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -974,7 +974,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>74</v>
+        <v>51</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -985,7 +985,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:48:48</t>
+          <t>06:11:46</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -999,7 +999,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1018,7 +1018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1031,14 +1031,66 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:48:48</t>
+          <t>Última actualización: 06:11:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>06:11:46</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>97</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4642
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:11:46</t>
+          <t>Última actualización: 06:43:29</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 23</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>06:11:46</t>
+          <t>06:43:29</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>06:11:46</t>
+          <t>06:43:29</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>06:11:46</t>
+          <t>06:43:29</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>75</v>
+        <v>38</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -753,16 +753,16 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>07:27</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>06:11:46</t>
+          <t>06:43:29</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>07:31</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>80</v>
+        <v>44</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,21 +798,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>06:11:46</t>
+          <t>06:43:29</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>85</v>
+        <v>47</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,21 +823,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>06:11:46</t>
+          <t>06:43:29</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>07:44</t>
+          <t>07:31</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>93</v>
+        <v>48</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,23 +848,198 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>06:11:46</t>
+          <t>06:43:29</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>53</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>06:43:29</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>07:44</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>61</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>06:43:29</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>07:51</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>68</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>06:43:29</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>08:01</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>78</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>06:43:29</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
           <t>08:06</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D21" t="n">
-        <v>115</v>
-      </c>
-      <c r="E21" t="inlineStr">
+      <c r="D25" t="n">
+        <v>83</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>06:43:29</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>08:19</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>96</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>06:43:29</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>98</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>06:43:29</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>08:25</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>102</v>
+      </c>
+      <c r="E28" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -881,7 +1056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -894,14 +1069,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:11:46</t>
+          <t>Última actualización: 06:43:29</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 4</t>
         </is>
       </c>
     </row>
@@ -960,7 +1135,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>06:11:46</t>
+          <t>06:43:29</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -974,7 +1149,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -985,7 +1160,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>06:11:46</t>
+          <t>06:43:29</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -999,9 +1174,34 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>80</v>
+        <v>48</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>06:43:29</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>07:51</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>68</v>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1018,7 +1218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1031,14 +1231,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:11:46</t>
+          <t>Última actualización: 06:43:29</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -1089,6 +1289,56 @@
         <v>97</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>06:43:29</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>07:49</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>66</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>06:43:29</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>08:38</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>115</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4643
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:43:29</t>
+          <t>Última actualización: 07:00:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 23</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>06:43:29</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>07:02</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>06:11:46</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>07:20</t>
+          <t>07:02</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>69</v>
+        <v>2</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,12 +723,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>06:43:29</t>
+          <t>06:11:46</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -737,7 +737,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>06:11:46</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>75</v>
+        <v>21</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>06:43:29</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>07:27</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,21 +798,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>06:43:29</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>47</v>
+        <v>27</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -828,16 +828,16 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>07:31</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -853,16 +853,16 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:31</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,21 +873,21 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>06:43:29</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>07:44</t>
+          <t>07:32</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>61</v>
+        <v>32</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -903,16 +903,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>07:51</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,21 +923,21 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>06:43:29</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>08:01</t>
+          <t>07:37</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>78</v>
+        <v>37</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -948,21 +948,21 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>06:43:29</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>08:06</t>
+          <t>07:44</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>83</v>
+        <v>44</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -973,21 +973,21 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>06:43:29</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>08:19</t>
+          <t>07:51</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>96</v>
+        <v>51</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,21 +998,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>06:43:29</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>98</v>
+        <v>61</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,23 +1023,173 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>07:00:10</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>08:06</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>66</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>07:00:10</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>08:19</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>79</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>07:00:10</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>81</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>06:43:29</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>08:25</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D28" t="n">
+      <c r="D31" t="n">
         <v>102</v>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>07:00:10</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>08:26</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>86</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>07:00:10</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>105</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>07:00:10</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>105</v>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1056,7 +1206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1069,14 +1219,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:43:29</t>
+          <t>Última actualización: 07:00:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -1135,7 +1285,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>06:43:29</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1149,7 +1299,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1185,23 +1335,98 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>06:43:29</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>07:32</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>32</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>07:00:10</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>07:51</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D9" t="n">
-        <v>68</v>
-      </c>
-      <c r="E9" t="inlineStr">
+      <c r="D10" t="n">
+        <v>51</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>07:00:10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>105</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>07:00:10</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>105</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1231,7 +1456,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:43:29</t>
+          <t>Última actualización: 07:00:10</t>
         </is>
       </c>
     </row>
@@ -1297,7 +1522,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>06:43:29</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1311,7 +1536,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>66</v>
+        <v>49</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1322,7 +1547,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>06:43:29</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1336,7 +1561,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>115</v>
+        <v>98</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4644
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:00:10</t>
+          <t>Última actualización: 07:24:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -773,12 +773,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>07:24:46</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>07:24</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -803,16 +803,16 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>07:27</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,21 +823,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>06:43:29</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>47</v>
+        <v>27</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -853,16 +853,16 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>07:31</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,12 +873,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>07:24:46</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>07:32</t>
+          <t>07:31</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -887,7 +887,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -898,21 +898,21 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>06:43:29</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:32</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>53</v>
+        <v>32</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,12 +923,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>07:24:46</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>07:37</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -937,7 +937,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -953,16 +953,16 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>07:44</t>
+          <t>07:37</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -973,21 +973,21 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>07:24:46</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>07:51</t>
+          <t>07:44</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,21 +998,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>07:24:46</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>08:01</t>
+          <t>07:51</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>61</v>
+        <v>27</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,21 +1023,21 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>07:24:46</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>08:06</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>66</v>
+        <v>37</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1048,21 +1048,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>07:24:46</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>08:19</t>
+          <t>08:06</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>79</v>
+        <v>42</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1073,21 +1073,21 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>07:24:46</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>08:19</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>81</v>
+        <v>55</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,21 +1098,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>06:43:29</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>08:25</t>
+          <t>08:21</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>102</v>
+        <v>81</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,12 +1123,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>07:24:46</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>08:26</t>
+          <t>08:25</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1137,7 +1137,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>86</v>
+        <v>61</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1153,16 +1153,16 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>08:26</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>105</v>
+        <v>86</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,23 +1173,223 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>07:24:46</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>80</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>07:24:46</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>80</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>07:00:10</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>08:45</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D34" t="n">
+      <c r="D36" t="n">
         <v>105</v>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>07:00:10</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>105</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>07:24:46</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>09:04</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>100</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>07:24:46</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>102</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>07:24:46</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>09:09</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>105</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>07:24:46</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>112</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>07:24:46</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>112</v>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1206,7 +1406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1219,14 +1419,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:00:10</t>
+          <t>Última actualización: 07:24:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -1310,7 +1510,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>06:43:29</t>
+          <t>07:24:46</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1324,7 +1524,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>48</v>
+        <v>7</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1360,7 +1560,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>07:24:46</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1374,7 +1574,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1385,12 +1585,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>07:24:46</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1399,7 +1599,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>105</v>
+        <v>80</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1410,23 +1610,98 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>07:24:46</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>80</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>07:00:10</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>08:45</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>105</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>07:00:10</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D14" t="n">
         <v>105</v>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>07:24:46</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>102</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1443,7 +1718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1456,14 +1731,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:00:10</t>
+          <t>Última actualización: 07:24:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -1497,7 +1772,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>06:11:46</t>
+          <t>07:24:46</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1511,7 +1786,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>97</v>
+        <v>24</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1547,25 +1822,75 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>07:24:46</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>08:37</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>73</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>07:00:10</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>08:38</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D9" t="n">
         <v>98</v>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>07:24:46</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>09:02</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>98</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4645
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:24:47</t>
+          <t>Última actualización: 07:46:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 44</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07:24:46</t>
+          <t>07:46:20</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1012,7 +1012,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1048,7 +1048,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>07:24:46</t>
+          <t>07:46:20</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1062,7 +1062,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1073,7 +1073,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>07:24:46</t>
+          <t>07:46:20</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1087,7 +1087,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>55</v>
+        <v>33</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>07:46:20</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1112,7 +1112,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>07:46:20</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>86</v>
+        <v>40</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,21 +1173,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>07:24:46</t>
+          <t>07:46:20</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>08:44</t>
+          <t>08:41</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1223,21 +1223,21 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>07:46:20</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>105</v>
+        <v>58</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>07:46:20</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>105</v>
+        <v>59</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,21 +1273,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07:24:46</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>09:04</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,21 +1298,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:24:46</t>
+          <t>07:46:20</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>102</v>
+        <v>78</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,21 +1323,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>07:24:46</t>
+          <t>07:46:20</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>09:09</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>105</v>
+        <v>80</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1353,16 +1353,16 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:09</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,23 +1373,198 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>07:46:20</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>09:10</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>84</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>07:46:20</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>90</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t>07:24:46</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t>09:16</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D42" t="n">
+      <c r="D44" t="n">
         <v>112</v>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>07:46:20</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>91</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>07:46:20</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>09:24</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>98</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>07:46:20</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>108</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>07:46:20</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>109</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>07:46:20</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>09:44</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>118</v>
+      </c>
+      <c r="E49" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1419,7 +1594,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:24:47</t>
+          <t>Última actualización: 07:46:20</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1735,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07:24:46</t>
+          <t>07:46:20</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1574,7 +1749,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1585,7 +1760,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>07:24:46</t>
+          <t>07:46:20</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1599,7 +1774,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>80</v>
+        <v>58</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1635,7 +1810,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>07:46:20</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1645,11 +1820,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>105</v>
+        <v>59</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1670,7 +1845,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1685,7 +1860,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>07:24:46</t>
+          <t>07:46:20</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1699,7 +1874,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>102</v>
+        <v>80</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1718,7 +1893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1731,14 +1906,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:24:47</t>
+          <t>Última actualización: 07:46:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -1772,12 +1947,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>07:24:46</t>
+          <t>07:46:20</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>07:48</t>
+          <t>07:47</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1786,7 +1961,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1797,12 +1972,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>07:24:46</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>07:49</t>
+          <t>07:48</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1811,7 +1986,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1822,12 +1997,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>07:24:46</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>08:37</t>
+          <t>07:49</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1836,7 +2011,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>73</v>
+        <v>49</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1847,12 +2022,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>07:24:46</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>08:38</t>
+          <t>08:37</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1861,7 +2036,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>98</v>
+        <v>73</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1872,23 +2047,73 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>07:46:20</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>08:38</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>52</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>07:24:46</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>09:02</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D11" t="n">
         <v>98</v>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>07:46:20</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>09:03</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>77</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4646
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:46:20</t>
+          <t>Última actualización: 08:00:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 44</t>
+          <t>Total filas: 46</t>
         </is>
       </c>
     </row>
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>07:24:46</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1048,7 +1048,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>07:46:20</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1062,7 +1062,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1073,7 +1073,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>07:46:20</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1087,7 +1087,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>07:46:20</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1112,7 +1112,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07:46:20</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>07:46:20</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1187,7 +1187,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1223,7 +1223,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>07:46:20</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1237,7 +1237,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>07:46:20</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1262,7 +1262,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:46:20</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1312,7 +1312,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,21 +1323,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>07:46:20</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>09:05</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,21 +1348,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>07:24:46</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>09:09</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>105</v>
+        <v>66</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,12 +1373,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:46:20</t>
+          <t>07:24:46</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>09:10</t>
+          <t>09:09</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>84</v>
+        <v>105</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1403,16 +1403,16 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:10</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07:24:46</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>112</v>
+        <v>76</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1453,16 +1453,16 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1478,16 +1478,16 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>09:24</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,21 +1498,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>07:46:20</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:24</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>108</v>
+        <v>84</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,21 +1523,21 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>07:46:20</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>09:35</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>109</v>
+        <v>94</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,23 +1548,73 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>07:46:20</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>95</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>08:00:25</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
           <t>09:44</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D49" t="n">
-        <v>118</v>
-      </c>
-      <c r="E49" t="inlineStr">
+      <c r="D50" t="n">
+        <v>104</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>08:00:25</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>115</v>
+      </c>
+      <c r="E51" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1581,7 +1631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1594,14 +1644,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:46:20</t>
+          <t>Última actualización: 08:00:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 11</t>
         </is>
       </c>
     </row>
@@ -1760,7 +1810,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>07:46:20</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1774,7 +1824,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1810,7 +1860,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>07:46:20</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1824,7 +1874,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1860,7 +1910,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>07:46:20</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1874,9 +1924,34 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>80</v>
+        <v>66</v>
       </c>
       <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>08:00:25</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>115</v>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1893,7 +1968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1906,14 +1981,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:46:20</t>
+          <t>Última actualización: 08:00:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -2047,7 +2122,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07:46:20</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2061,7 +2136,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -2097,7 +2172,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>07:46:20</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2111,11 +2186,36 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>08:00:25</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>09:28</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>88</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4647
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:00:25</t>
+          <t>Última actualización: 08:29:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 46</t>
+          <t>Total filas: 54</t>
         </is>
       </c>
     </row>
@@ -1173,21 +1173,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>08:41</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>41</v>
+        <v>1</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,21 +1198,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>07:24:46</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>08:44</t>
+          <t>08:41</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>80</v>
+        <v>12</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1223,7 +1223,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1237,7 +1237,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>44</v>
+        <v>15</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1248,12 +1248,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1262,7 +1262,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1303,16 +1303,16 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>09:04</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>64</v>
+        <v>45</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,21 +1323,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>09:05</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>65</v>
+        <v>35</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1353,16 +1353,16 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>09:05</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,21 +1373,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:24:46</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>09:09</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>105</v>
+        <v>37</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,12 +1398,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:46:20</t>
+          <t>07:24:46</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>09:10</t>
+          <t>09:09</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1412,7 +1412,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>84</v>
+        <v>105</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,21 +1423,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>07:46:20</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:10</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,21 +1448,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>07:46:20</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>90</v>
+        <v>42</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,12 +1473,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>07:46:20</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>91</v>
+        <v>76</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,21 +1498,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>09:24</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>84</v>
+        <v>47</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,21 +1523,21 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>07:46:20</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,21 +1548,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>09:35</t>
+          <t>09:24</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>95</v>
+        <v>55</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,21 +1573,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>09:44</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>104</v>
+        <v>65</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,23 +1598,223 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t>08:29:38</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>66</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>08:29:38</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>09:44</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>75</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>08:29:38</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>09:54</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>85</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
           <t>08:00:25</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>09:55</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D51" t="n">
+      <c r="D54" t="n">
         <v>115</v>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>08:29:38</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>10:01</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>92</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>08:29:38</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>95</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>08:29:38</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>106</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>08:29:38</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>10:16</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>107</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>08:29:38</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>10:24</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>115</v>
+      </c>
+      <c r="E59" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1631,7 +1831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1644,14 +1844,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:00:25</t>
+          <t>Última actualización: 08:29:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 11</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -1810,7 +2010,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1824,7 +2024,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>44</v>
+        <v>15</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1835,7 +2035,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>07:24:46</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1849,7 +2049,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>80</v>
+        <v>15</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1910,7 +2110,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1924,7 +2124,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>66</v>
+        <v>37</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1935,23 +2135,48 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>08:29:38</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>09:54</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>85</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>08:00:25</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>09:55</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D16" t="n">
+      <c r="D17" t="n">
         <v>115</v>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1968,7 +2193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1981,14 +2206,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:00:25</t>
+          <t>Última actualización: 08:29:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -2097,7 +2322,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>07:24:46</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2111,7 +2336,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>73</v>
+        <v>8</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -2147,7 +2372,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>07:24:46</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2161,7 +2386,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>98</v>
+        <v>33</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -2197,25 +2422,75 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>08:29:38</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>09:27</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>58</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>08:00:25</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>09:28</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="D14" t="n">
         <v>88</v>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>08:29:38</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>10:17</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>108</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4648
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:29:38</t>
+          <t>Última actualización: 08:50:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 54</t>
+          <t>Total filas: 61</t>
         </is>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1323,12 +1323,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>09:04</t>
+          <t>09:03</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,21 +1348,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>09:05</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>65</v>
+        <v>35</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,21 +1373,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>09:05</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>37</v>
+        <v>65</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,21 +1398,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:24:46</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>09:09</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>105</v>
+        <v>16</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,12 +1423,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07:46:20</t>
+          <t>07:24:46</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>09:10</t>
+          <t>09:09</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>84</v>
+        <v>105</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,12 +1448,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>07:46:20</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>09:11</t>
+          <t>09:10</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1462,7 +1462,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>42</v>
+        <v>84</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,21 +1473,21 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>76</v>
+        <v>21</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1508,11 +1508,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>47</v>
+        <v>26</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,21 +1523,21 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>07:46:20</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>91</v>
+        <v>26</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,21 +1548,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>07:46:20</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>09:24</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>55</v>
+        <v>91</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,21 +1573,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:23</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>65</v>
+        <v>33</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1603,16 +1603,16 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>09:35</t>
+          <t>09:24</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1623,21 +1623,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>09:44</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>75</v>
+        <v>44</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1648,21 +1648,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>09:54</t>
+          <t>09:35</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>85</v>
+        <v>45</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,21 +1673,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>09:55</t>
+          <t>09:44</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,21 +1698,21 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>10:01</t>
+          <t>09:54</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>92</v>
+        <v>64</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,21 +1723,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>10:04</t>
+          <t>09:55</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>95</v>
+        <v>115</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1753,16 +1753,16 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1773,21 +1773,21 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>10:16</t>
+          <t>10:03</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>107</v>
+        <v>73</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,23 +1798,198 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
+          <t>08:50:55</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>74</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
           <t>08:29:38</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>95</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>08:50:55</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>85</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>08:29:38</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>10:16</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>107</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>08:50:55</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
         <is>
           <t>10:24</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C63" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D59" t="n">
-        <v>115</v>
-      </c>
-      <c r="E59" t="inlineStr">
+      <c r="D63" t="n">
+        <v>94</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>08:50:55</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>10:26</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>96</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>08:50:55</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>104</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>08:50:55</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>113</v>
+      </c>
+      <c r="E66" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1844,7 +2019,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:29:38</t>
+          <t>Última actualización: 08:50:55</t>
         </is>
       </c>
     </row>
@@ -2110,7 +2285,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2124,7 +2299,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2135,7 +2310,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2149,7 +2324,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>85</v>
+        <v>64</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -2193,7 +2368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2206,14 +2381,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:29:38</t>
+          <t>Última actualización: 08:50:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -2372,7 +2547,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2386,7 +2561,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -2422,7 +2597,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2436,7 +2611,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>58</v>
+        <v>37</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -2472,7 +2647,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2486,11 +2661,61 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>108</v>
+        <v>87</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>08:50:55</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>10:29</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>99</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>08:50:55</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>10:42</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>112</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4649
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E66"/>
+  <dimension ref="A1:E73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:50:55</t>
+          <t>Última actualización: 08:58:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 61</t>
+          <t>Total filas: 68</t>
         </is>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1323,12 +1323,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>09:03</t>
+          <t>09:01</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,12 +1348,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>09:04</t>
+          <t>09:03</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1362,7 +1362,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,21 +1373,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>09:05</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>65</v>
+        <v>35</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,21 +1398,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>09:05</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>16</v>
+        <v>65</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,21 +1423,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07:24:46</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>09:09</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>105</v>
+        <v>8</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,12 +1448,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>07:46:20</t>
+          <t>07:24:46</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>09:10</t>
+          <t>09:09</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1462,7 +1462,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>84</v>
+        <v>105</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,12 +1473,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>07:46:20</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>09:11</t>
+          <t>09:10</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>21</v>
+        <v>84</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,21 +1498,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1537,7 +1537,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,12 +1548,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>07:46:20</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>91</v>
+        <v>26</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,21 +1573,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>09:23</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,12 +1598,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>09:24</t>
+          <t>09:23</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>55</v>
+        <v>33</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1623,21 +1623,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:24</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1648,21 +1648,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>09:35</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,21 +1673,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>09:44</t>
+          <t>09:35</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1703,16 +1703,16 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>09:54</t>
+          <t>09:44</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,21 +1723,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>09:55</t>
+          <t>09:45</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>115</v>
+        <v>47</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,21 +1748,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>10:01</t>
+          <t>09:54</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>92</v>
+        <v>64</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1773,21 +1773,21 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>10:03</t>
+          <t>09:55</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>73</v>
+        <v>57</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,12 +1798,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>10:04</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -1812,7 +1812,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,21 +1823,21 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>10:04</t>
+          <t>10:03</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>95</v>
+        <v>65</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1853,16 +1853,16 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>10:03</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,21 +1873,21 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>10:16</t>
+          <t>10:04</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>107</v>
+        <v>66</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1903,16 +1903,16 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>10:24</t>
+          <t>10:04</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>94</v>
+        <v>74</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,21 +1923,21 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>10:26</t>
+          <t>10:15</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,21 +1948,21 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>10:34</t>
+          <t>10:16</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1978,18 +1978,193 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
+          <t>10:24</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>94</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>08:58:16</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>10:25</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>87</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>08:58:16</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>10:26</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>88</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>08:58:16</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>96</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>08:50:55</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
           <t>10:43</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C70" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D66" t="n">
+      <c r="D70" t="n">
         <v>113</v>
       </c>
-      <c r="E66" t="inlineStr">
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>08:58:16</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>106</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>08:58:16</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>117</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>08:58:16</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>10:57</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>119</v>
+      </c>
+      <c r="E73" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2019,7 +2194,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:50:55</t>
+          <t>Última actualización: 08:58:16</t>
         </is>
       </c>
     </row>
@@ -2285,7 +2460,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2299,7 +2474,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2335,7 +2510,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2349,7 +2524,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>115</v>
+        <v>57</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -2368,7 +2543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2381,14 +2556,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:50:55</t>
+          <t>Última actualización: 08:58:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -2572,7 +2747,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2586,7 +2761,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>63</v>
+        <v>5</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2622,7 +2797,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2636,7 +2811,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>88</v>
+        <v>30</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2672,25 +2847,25 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>10:29</t>
+          <t>10:18</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
@@ -2702,18 +2877,93 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>10:29</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>99</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>08:58:16</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>92</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>08:50:55</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
           <t>10:42</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D17" t="n">
+      <c r="D19" t="n">
         <v>112</v>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>08:58:16</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>105</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4650
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E73"/>
+  <dimension ref="A1:E81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:58:16</t>
+          <t>Última actualización: 09:31:22</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 68</t>
+          <t>Total filas: 76</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>105</v>
+        <v>45</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>45</v>
+        <v>105</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1648,7 +1648,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1662,7 +1662,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1748,21 +1748,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>09:54</t>
+          <t>09:51</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>64</v>
+        <v>20</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1773,12 +1773,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>09:55</t>
+          <t>09:54</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,21 +1798,21 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>10:01</t>
+          <t>09:55</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>92</v>
+        <v>24</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,21 +1823,21 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>10:03</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,21 +1848,21 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>10:03</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>73</v>
+        <v>30</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1878,16 +1878,16 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>10:04</t>
+          <t>10:03</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1903,16 +1903,16 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>10:04</t>
+          <t>10:03</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,21 +1923,21 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>10:04</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,21 +1948,21 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>10:16</t>
+          <t>10:04</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>107</v>
+        <v>33</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,21 +1973,21 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>10:24</t>
+          <t>10:15</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>94</v>
+        <v>44</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,21 +1998,21 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>10:25</t>
+          <t>10:16</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>87</v>
+        <v>107</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,21 +2023,21 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>10:26</t>
+          <t>10:24</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2053,16 +2053,16 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>10:34</t>
+          <t>10:25</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,21 +2073,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>10:43</t>
+          <t>10:26</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>113</v>
+        <v>88</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,21 +2098,21 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>10:44</t>
+          <t>10:34</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>106</v>
+        <v>63</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2123,21 +2123,21 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>10:55</t>
+          <t>10:43</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,23 +2148,223 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>73</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>09:31:22</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>80</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>09:31:22</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>84</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>09:31:22</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
           <t>10:57</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
+      <c r="C76" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D73" t="n">
-        <v>119</v>
-      </c>
-      <c r="E73" t="inlineStr">
+      <c r="D76" t="n">
+        <v>86</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>09:31:22</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>11:04</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>93</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>09:31:22</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>11:08</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>97</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>09:31:22</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>104</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>09:31:22</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>11:24</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>113</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>09:31:22</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>11:28</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>117</v>
+      </c>
+      <c r="E81" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2194,7 +2394,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:58:16</t>
+          <t>Última actualización: 09:31:22</t>
         </is>
       </c>
     </row>
@@ -2510,7 +2710,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2524,7 +2724,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -2543,7 +2743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2556,14 +2756,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:58:16</t>
+          <t>Última actualización: 09:31:22</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -2822,37 +3022,37 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10:17</t>
+          <t>09:33</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>87</v>
+        <v>2</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>10:18</t>
+          <t>10:17</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2861,7 +3061,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -2872,37 +3072,37 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>10:29</t>
+          <t>10:18</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>99</v>
+        <v>47</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>10:29</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2911,7 +3111,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -2922,21 +3122,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>10:42</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>112</v>
+        <v>59</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -2947,25 +3147,75 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>10:42</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>112</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>09:31:22</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
           <t>10:43</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D20" t="n">
-        <v>105</v>
-      </c>
-      <c r="E20" t="inlineStr">
+      <c r="D21" t="n">
+        <v>72</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>09:31:22</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>11:23</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>112</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4651
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E81"/>
+  <dimension ref="A1:E92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:31:22</t>
+          <t>Última actualización: 10:16:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 76</t>
+          <t>Total filas: 87</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,21 +2023,21 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>10:24</t>
+          <t>10:16</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,12 +2048,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>10:25</t>
+          <t>10:24</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2062,7 +2062,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,21 +2073,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>10:26</t>
+          <t>10:25</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>88</v>
+        <v>9</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,21 +2098,21 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>10:34</t>
+          <t>10:26</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2123,21 +2123,21 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>10:43</t>
+          <t>10:34</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>113</v>
+        <v>18</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,21 +2148,21 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>10:44</t>
+          <t>10:42</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>73</v>
+        <v>26</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,21 +2173,21 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>10:51</t>
+          <t>10:43</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>80</v>
+        <v>113</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,21 +2198,21 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>10:55</t>
+          <t>10:44</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>84</v>
+        <v>28</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2223,21 +2223,21 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>10:57</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>86</v>
+        <v>35</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,21 +2248,21 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>11:04</t>
+          <t>10:55</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>93</v>
+        <v>39</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2278,16 +2278,16 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>11:08</t>
+          <t>10:57</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2298,21 +2298,21 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>11:15</t>
+          <t>11:01</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>104</v>
+        <v>45</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,21 +2323,21 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>11:24</t>
+          <t>11:04</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>113</v>
+        <v>48</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,23 +2348,298 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
+          <t>10:16:16</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>11:08</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>52</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>10:16:16</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>59</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>10:16:16</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>11:24</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>68</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
           <t>09:31:22</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr">
+      <c r="B84" t="inlineStr">
         <is>
           <t>11:28</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
+      <c r="C84" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D81" t="n">
+      <c r="D84" t="n">
         <v>117</v>
       </c>
-      <c r="E81" t="inlineStr">
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>10:16:16</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>78</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>10:16:16</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>79</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>10:16:16</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>11:43</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>87</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>10:16:16</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>89</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>10:16:16</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>11:54</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>98</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>10:16:16</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>99</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>10:16:16</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>12:04</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>108</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>10:16:16</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>119</v>
+      </c>
+      <c r="E92" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2381,7 +2656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2394,14 +2669,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:31:22</t>
+          <t>Última actualización: 10:16:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -2727,6 +3002,56 @@
         <v>24</v>
       </c>
       <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>10:16:16</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>79</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>10:16:16</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>89</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2756,7 +3081,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:31:22</t>
+          <t>Última actualización: 10:16:16</t>
         </is>
       </c>
     </row>
@@ -3047,7 +3372,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -3061,7 +3386,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>87</v>
+        <v>1</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -3122,7 +3447,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3136,7 +3461,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>59</v>
+        <v>14</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -3172,7 +3497,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3186,7 +3511,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>72</v>
+        <v>27</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -3197,7 +3522,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3211,7 +3536,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>112</v>
+        <v>67</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4652
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E92"/>
+  <dimension ref="A1:E99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:16:16</t>
+          <t>Última actualización: 10:46:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 87</t>
+          <t>Total filas: 94</t>
         </is>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -2223,7 +2223,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>10:46:10</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2237,7 +2237,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>35</v>
+        <v>5</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>10:46:10</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2262,7 +2262,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>10:46:10</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>86</v>
+        <v>11</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2298,7 +2298,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>10:46:10</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2312,7 +2312,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2348,21 +2348,21 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>10:46:10</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>11:08</t>
+          <t>11:05</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>52</v>
+        <v>19</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,21 +2373,21 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>10:46:10</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>11:15</t>
+          <t>11:08</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>59</v>
+        <v>22</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,21 +2398,21 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>10:46:10</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>11:24</t>
+          <t>11:15</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>68</v>
+        <v>29</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,21 +2423,21 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>10:46:10</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>11:28</t>
+          <t>11:24</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>117</v>
+        <v>38</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2448,21 +2448,21 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>11:34</t>
+          <t>11:28</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>78</v>
+        <v>117</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2478,16 +2478,16 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>11:35</t>
+          <t>11:34</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,21 +2498,21 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>10:46:10</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>11:43</t>
+          <t>11:35</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>87</v>
+        <v>49</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,21 +2523,21 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>10:46:10</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>11:45</t>
+          <t>11:36</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>89</v>
+        <v>50</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2553,16 +2553,16 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>11:54</t>
+          <t>11:43</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2573,21 +2573,21 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>10:46:10</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>11:55</t>
+          <t>11:45</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>99</v>
+        <v>59</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2598,21 +2598,21 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>10:46:10</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>12:04</t>
+          <t>11:45</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>108</v>
+        <v>59</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,23 +2623,198 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>10:46:10</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
+          <t>11:54</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>68</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>10:46:10</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>69</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>10:46:10</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>12:04</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>78</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>10:46:10</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr">
+      <c r="C95" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D92" t="n">
-        <v>119</v>
-      </c>
-      <c r="E92" t="inlineStr">
+      <c r="D95" t="n">
+        <v>89</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>10:46:10</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>99</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>10:46:10</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>108</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>10:46:10</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>12:37</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>111</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>10:46:10</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>12:44</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>118</v>
+      </c>
+      <c r="E99" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2669,7 +2844,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:16:16</t>
+          <t>Última actualización: 10:46:10</t>
         </is>
       </c>
     </row>
@@ -3010,7 +3185,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>10:46:10</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3024,7 +3199,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>79</v>
+        <v>49</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -3035,7 +3210,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>10:46:10</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3049,7 +3224,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>89</v>
+        <v>59</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -3068,7 +3243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3081,14 +3256,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:16:16</t>
+          <t>Última actualización: 10:46:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -3522,23 +3697,48 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>10:46:10</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>10:46</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>10:46:10</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
           <t>11:23</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D22" t="n">
-        <v>67</v>
-      </c>
-      <c r="E22" t="inlineStr">
+      <c r="D23" t="n">
+        <v>37</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4653
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E99"/>
+  <dimension ref="A1:E103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:46:10</t>
+          <t>Última actualización: 11:01:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 94</t>
+          <t>Total filas: 98</t>
         </is>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1533,11 +1533,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -2348,7 +2348,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>11:01:03</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2362,7 +2362,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>11:01:03</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2387,7 +2387,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>11:01:03</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2412,7 +2412,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>11:01:03</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2437,7 +2437,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>11:01:03</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2512,7 +2512,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>11:01:03</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2537,7 +2537,7 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2548,12 +2548,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>11:01:03</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>11:43</t>
+          <t>11:42</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -2562,7 +2562,7 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>87</v>
+        <v>41</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2573,21 +2573,21 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>11:45</t>
+          <t>11:43</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>59</v>
+        <v>87</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>11:01:03</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2628,16 +2628,16 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>11:54</t>
+          <t>11:45</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2648,21 +2648,21 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>11:01:03</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>11:55</t>
+          <t>11:54</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>69</v>
+        <v>53</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2673,21 +2673,21 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>11:01:03</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>12:04</t>
+          <t>11:55</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>78</v>
+        <v>54</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,21 +2698,21 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>11:01:03</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>12:04</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>89</v>
+        <v>63</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,21 +2723,21 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>11:01:03</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>12:25</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>99</v>
+        <v>74</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,21 +2748,21 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>11:01:03</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>108</v>
+        <v>84</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,21 +2773,21 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>11:01:03</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>12:37</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>111</v>
+        <v>89</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,23 +2798,123 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>11:01:03</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>93</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>11:01:03</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>12:37</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>96</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>11:01:03</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
           <t>12:44</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr">
+      <c r="C101" t="inlineStr">
         <is>
           <t>14X44_ABASTO</t>
         </is>
       </c>
-      <c r="D99" t="n">
-        <v>118</v>
-      </c>
-      <c r="E99" t="inlineStr">
+      <c r="D101" t="n">
+        <v>103</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>11:01:03</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>12:46</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>105</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>11:01:03</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>114</v>
+      </c>
+      <c r="E103" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2831,7 +2931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2844,14 +2944,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:46:10</t>
+          <t>Última actualización: 11:01:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -3185,7 +3285,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>11:01:03</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3199,7 +3299,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -3210,7 +3310,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>11:01:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3224,9 +3324,34 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>11:01:03</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>114</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3256,7 +3381,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:46:10</t>
+          <t>Última actualización: 11:01:03</t>
         </is>
       </c>
     </row>
@@ -3722,7 +3847,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>11:01:03</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3736,7 +3861,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4654
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E103"/>
+  <dimension ref="A1:E109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:01:03</t>
+          <t>Última actualización: 11:33:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 98</t>
+          <t>Total filas: 104</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>45</v>
+        <v>105</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>105</v>
+        <v>45</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>11:01:03</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2512,7 +2512,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>11:01:03</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2537,7 +2537,7 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2573,7 +2573,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2587,7 +2587,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>87</v>
+        <v>10</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>11:01:03</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2612,7 +2612,7 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2648,7 +2648,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>11:01:03</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2662,7 +2662,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>53</v>
+        <v>21</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>11:01:03</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2687,7 +2687,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>11:01:03</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2712,7 +2712,7 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>63</v>
+        <v>31</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>11:01:03</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2737,7 +2737,7 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>74</v>
+        <v>42</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>11:01:03</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2762,7 +2762,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>84</v>
+        <v>52</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,12 +2773,12 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>11:01:03</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>12:28</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -2787,7 +2787,7 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>89</v>
+        <v>55</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2803,16 +2803,16 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,21 +2823,21 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>11:01:03</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>12:37</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>96</v>
+        <v>61</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,21 +2848,21 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>11:01:03</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>12:44</t>
+          <t>12:35</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>103</v>
+        <v>62</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2878,16 +2878,16 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>12:46</t>
+          <t>12:37</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>105</v>
+        <v>96</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,23 +2898,173 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>11:01:03</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
+          <t>12:44</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>71</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>11:33:07</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>12:46</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>73</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>11:33:07</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
           <t>12:55</t>
         </is>
       </c>
-      <c r="C103" t="inlineStr">
+      <c r="C105" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D103" t="n">
-        <v>114</v>
-      </c>
-      <c r="E103" t="inlineStr">
+      <c r="D105" t="n">
+        <v>82</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>11:33:07</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>13:05</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>92</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>11:33:07</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>102</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>11:33:07</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>111</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>11:33:07</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>119</v>
+      </c>
+      <c r="E109" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2931,7 +3081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2944,14 +3094,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:01:03</t>
+          <t>Última actualización: 11:33:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -3120,7 +3270,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -3145,7 +3295,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -3285,7 +3435,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>11:01:03</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3299,7 +3449,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -3310,7 +3460,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>11:01:03</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3324,7 +3474,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -3335,7 +3485,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>11:01:03</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3349,9 +3499,34 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>114</v>
+        <v>82</v>
       </c>
       <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>11:33:07</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>119</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3368,7 +3543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3381,14 +3556,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:01:03</t>
+          <t>Última actualización: 11:33:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -3864,6 +4039,31 @@
         <v>22</v>
       </c>
       <c r="E23" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>11:33:07</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>13:23</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>110</v>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4655
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E109"/>
+  <dimension ref="A1:E121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:33:07</t>
+          <t>Última actualización: 11:53:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 104</t>
+          <t>Total filas: 116</t>
         </is>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>105</v>
+        <v>45</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>45</v>
+        <v>105</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>10:46:10</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>12</v>
+        <v>59</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2633,11 +2633,11 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>59</v>
+        <v>12</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2648,7 +2648,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2662,7 +2662,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2687,7 +2687,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,12 +2698,12 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>12:04</t>
+          <t>12:03</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -2712,7 +2712,7 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2728,16 +2728,16 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>12:04</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,21 +2748,21 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>12:25</t>
+          <t>12:11</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,21 +2773,21 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>12:28</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>55</v>
+        <v>22</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,21 +2798,21 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>11:01:03</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>89</v>
+        <v>31</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2828,16 +2828,16 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,12 +2848,12 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>12:35</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -2862,7 +2862,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>62</v>
+        <v>32</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,21 +2873,21 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>11:01:03</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>12:37</t>
+          <t>12:28</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>96</v>
+        <v>55</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,21 +2898,21 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>11:01:03</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>12:44</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,21 +2923,21 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>12:46</t>
+          <t>12:31</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>73</v>
+        <v>38</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,21 +2948,21 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>82</v>
+        <v>41</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2978,16 +2978,16 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>13:05</t>
+          <t>12:35</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>92</v>
+        <v>62</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,21 +2998,21 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>11:01:03</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>12:37</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,21 +3023,21 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>12:43</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3053,18 +3053,318 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
+          <t>12:44</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>71</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>11:53:55</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>12:46</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>53</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>11:53:55</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>12:54</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>61</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>11:33:07</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>82</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>11:53:55</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>13:04</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>71</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>11:33:07</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>13:05</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>92</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>11:53:55</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>82</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>11:53:55</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>13:23</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>90</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>11:53:55</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>91</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>11:33:07</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>111</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>11:53:55</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>98</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>11:33:07</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
           <t>13:32</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr">
+      <c r="C120" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D109" t="n">
+      <c r="D120" t="n">
         <v>119</v>
       </c>
-      <c r="E109" t="inlineStr">
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>11:53:55</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>13:44</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>111</v>
+      </c>
+      <c r="E121" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3081,7 +3381,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3094,14 +3394,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:33:07</t>
+          <t>Última actualización: 11:53:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -3310,7 +3610,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -3320,11 +3620,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>45</v>
+        <v>105</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -3335,7 +3635,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -3345,11 +3645,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>105</v>
+        <v>45</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -3485,12 +3785,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:54</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3499,7 +3799,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -3515,18 +3815,68 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>82</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>11:53:55</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>98</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>11:33:07</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
           <t>13:32</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D21" t="n">
+      <c r="D23" t="n">
         <v>119</v>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3543,7 +3893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3556,14 +3906,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:33:07</t>
+          <t>Última actualización: 11:53:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 21</t>
         </is>
       </c>
     </row>
@@ -4047,25 +4397,75 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>11:53:55</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>13:22</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>89</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>11:33:07</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>13:23</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D24" t="n">
+      <c r="D25" t="n">
         <v>110</v>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>11:53:55</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>13:49</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>116</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4656
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E121"/>
+  <dimension ref="A1:E129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:53:55</t>
+          <t>Última actualización: 12:10:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 116</t>
+          <t>Total filas: 124</t>
         </is>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>33</v>
+        <v>74</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>59</v>
+        <v>12</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>10:46:10</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2633,11 +2633,11 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>12</v>
+        <v>59</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2748,12 +2748,12 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>12:11</t>
+          <t>12:10</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -2762,7 +2762,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2778,16 +2778,16 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>12:11</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,21 +2798,21 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>12:24</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>31</v>
+        <v>5</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,21 +2823,21 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>12:25</t>
+          <t>12:23</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>52</v>
+        <v>13</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2853,16 +2853,16 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>12:25</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,21 +2873,21 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>12:28</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>55</v>
+        <v>15</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,21 +2898,21 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>11:01:03</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>89</v>
+        <v>32</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,12 +2923,12 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>12:31</t>
+          <t>12:28</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -2937,7 +2937,7 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,21 +2948,21 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>11:01:03</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>41</v>
+        <v>89</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,21 +2973,21 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>12:35</t>
+          <t>12:31</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>62</v>
+        <v>38</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,21 +2998,21 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>11:01:03</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>12:37</t>
+          <t>12:32</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>96</v>
+        <v>22</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,21 +3023,21 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>12:43</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3053,16 +3053,16 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>12:44</t>
+          <t>12:35</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,21 +3073,21 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>11:01:03</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>12:46</t>
+          <t>12:37</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>53</v>
+        <v>96</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3103,16 +3103,16 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>12:54</t>
+          <t>12:43</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,21 +3123,21 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:44</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>82</v>
+        <v>34</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3148,21 +3148,21 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>13:04</t>
+          <t>12:46</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>71</v>
+        <v>36</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3173,21 +3173,21 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>13:05</t>
+          <t>12:54</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>92</v>
+        <v>61</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,21 +3198,21 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>82</v>
+        <v>45</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3228,16 +3228,16 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>13:23</t>
+          <t>13:04</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>90</v>
+        <v>71</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,21 +3248,21 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:05</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>91</v>
+        <v>55</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,21 +3273,21 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>111</v>
+        <v>65</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3303,16 +3303,16 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>13:31</t>
+          <t>13:23</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,21 +3323,21 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>119</v>
+        <v>74</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3353,18 +3353,218 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>91</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>12:10:06</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>81</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>11:53:55</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>98</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>12:10:06</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>82</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>11:53:55</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
           <t>13:44</t>
         </is>
       </c>
-      <c r="C121" t="inlineStr">
+      <c r="C125" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D121" t="n">
+      <c r="D125" t="n">
         <v>111</v>
       </c>
-      <c r="E121" t="inlineStr">
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>12:10:06</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>95</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>12:10:06</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>105</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>12:10:06</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>14:03</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>113</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>12:10:06</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>14:04</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>114</v>
+      </c>
+      <c r="E129" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3394,7 +3594,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:53:55</t>
+          <t>Última actualización: 12:10:06</t>
         </is>
       </c>
     </row>
@@ -3810,7 +4010,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3824,7 +4024,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>82</v>
+        <v>45</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -3860,7 +4060,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3874,7 +4074,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>119</v>
+        <v>82</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -3893,7 +4093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3906,14 +4106,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:53:55</t>
+          <t>Última actualización: 12:10:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 21</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -4422,7 +4622,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -4436,7 +4636,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>110</v>
+        <v>73</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -4464,6 +4664,31 @@
         <v>116</v>
       </c>
       <c r="E26" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>12:10:06</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>100</v>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4657
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E129"/>
+  <dimension ref="A1:E138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:10:06</t>
+          <t>Última actualización: 12:33:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 124</t>
+          <t>Total filas: 133</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -3023,21 +3023,21 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:33</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,21 +3048,21 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>12:35</t>
+          <t>12:33</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,21 +3073,21 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>11:01:03</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>12:37</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>96</v>
+        <v>1</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3098,21 +3098,21 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>12:43</t>
+          <t>12:35</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,21 +3123,21 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>11:01:03</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>12:44</t>
+          <t>12:37</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>34</v>
+        <v>96</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3148,21 +3148,21 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>12:46</t>
+          <t>12:43</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3173,21 +3173,21 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>12:54</t>
+          <t>12:44</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>61</v>
+        <v>11</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3203,16 +3203,16 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:46</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,21 +3223,21 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>13:04</t>
+          <t>12:54</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>71</v>
+        <v>21</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3253,16 +3253,16 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>13:05</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,21 +3273,21 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>13:04</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>65</v>
+        <v>31</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3298,21 +3298,21 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>13:23</t>
+          <t>13:05</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>90</v>
+        <v>55</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,21 +3323,21 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>74</v>
+        <v>42</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3353,16 +3353,16 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:23</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,12 +3373,12 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>13:31</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -3387,7 +3387,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,21 +3398,21 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>13:31</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>98</v>
+        <v>51</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,21 +3423,21 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:27</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>82</v>
+        <v>54</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,21 +3448,21 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>13:44</t>
+          <t>13:31</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>111</v>
+        <v>58</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3478,16 +3478,16 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>13:45</t>
+          <t>13:31</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3503,16 +3503,16 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>105</v>
+        <v>82</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,21 +3523,21 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>14:03</t>
+          <t>13:44</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>113</v>
+        <v>71</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3553,18 +3553,243 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>95</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>12:33:46</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>82</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>12:33:46</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>83</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>12:10:06</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>14:03</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>113</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>12:33:46</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
           <t>14:04</t>
         </is>
       </c>
-      <c r="C129" t="inlineStr">
+      <c r="C133" t="inlineStr">
         <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D129" t="n">
-        <v>114</v>
-      </c>
-      <c r="E129" t="inlineStr">
+      <c r="D133" t="n">
+        <v>91</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>12:33:46</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>14:13</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>100</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>12:33:46</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>101</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>12:33:46</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>101</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>12:33:46</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>14:24</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>111</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>12:33:46</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>14:31</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>118</v>
+      </c>
+      <c r="E138" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3594,7 +3819,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:10:06</t>
+          <t>Última actualización: 12:33:46</t>
         </is>
       </c>
     </row>
@@ -3985,7 +4210,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3999,7 +4224,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>61</v>
+        <v>21</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -4035,7 +4260,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -4049,7 +4274,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>98</v>
+        <v>58</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -4106,7 +4331,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:10:06</t>
+          <t>Última actualización: 12:33:46</t>
         </is>
       </c>
     </row>
@@ -4597,7 +4822,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4611,7 +4836,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>89</v>
+        <v>49</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -4647,7 +4872,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -4661,7 +4886,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>116</v>
+        <v>76</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4658
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E138"/>
+  <dimension ref="A1:E145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:33:46</t>
+          <t>Última actualización: 12:52:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 133</t>
+          <t>Total filas: 140</t>
         </is>
       </c>
     </row>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1533,11 +1533,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>33</v>
+        <v>74</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>10:46:10</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>12</v>
+        <v>59</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2633,11 +2633,11 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>59</v>
+        <v>12</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3262,7 +3262,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>45</v>
+        <v>3</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3298,7 +3298,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>55</v>
+        <v>13</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3337,7 +3337,7 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,21 +3348,21 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>13:23</t>
+          <t>13:22</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3378,16 +3378,16 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:23</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,7 +3398,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3408,11 +3408,11 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>51</v>
+        <v>91</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,21 +3423,21 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>13:27</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3453,16 +3453,16 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>13:31</t>
+          <t>13:27</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3503,16 +3503,16 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:31</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,21 +3523,21 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>13:44</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>71</v>
+        <v>40</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,12 +3548,12 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>13:45</t>
+          <t>13:44</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -3562,7 +3562,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>95</v>
+        <v>71</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,21 +3573,21 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>13:45</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>82</v>
+        <v>53</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,21 +3598,21 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>13:56</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>83</v>
+        <v>63</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,21 +3623,21 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>14:03</t>
+          <t>13:56</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>113</v>
+        <v>64</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,21 +3648,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>14:04</t>
+          <t>14:03</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>91</v>
+        <v>113</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,21 +3673,21 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>14:13</t>
+          <t>14:04</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>100</v>
+        <v>72</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,21 +3698,21 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:12</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>101</v>
+        <v>80</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3728,16 +3728,16 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:13</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,21 +3748,21 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>111</v>
+        <v>82</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,23 +3773,198 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
+          <t>12:52:01</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>82</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>12:52:01</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>83</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>12:52:01</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>85</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
           <t>12:33:46</t>
         </is>
       </c>
-      <c r="B138" t="inlineStr">
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>14:24</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>111</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>12:52:01</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>93</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>12:52:01</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
         <is>
           <t>14:31</t>
         </is>
       </c>
-      <c r="C138" t="inlineStr">
+      <c r="C143" t="inlineStr">
         <is>
           <t>16_SANTA ANA</t>
         </is>
       </c>
-      <c r="D138" t="n">
-        <v>118</v>
-      </c>
-      <c r="E138" t="inlineStr">
+      <c r="D143" t="n">
+        <v>99</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>12:52:01</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>103</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>12:52:01</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>14:44</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>112</v>
+      </c>
+      <c r="E145" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3806,7 +3981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3819,14 +3994,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:33:46</t>
+          <t>Última actualización: 12:52:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -4235,7 +4410,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -4249,7 +4424,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>45</v>
+        <v>3</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -4285,7 +4460,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4299,9 +4474,34 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>82</v>
+        <v>40</v>
       </c>
       <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>12:52:01</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>103</v>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4318,7 +4518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4331,14 +4531,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:33:46</t>
+          <t>Última actualización: 12:52:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 23</t>
         </is>
       </c>
     </row>
@@ -4847,7 +5047,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -4861,7 +5061,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>73</v>
+        <v>31</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -4897,7 +5097,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -4911,11 +5111,36 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>100</v>
+        <v>58</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>12:52:01</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>14:43</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>111</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4659
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E145"/>
+  <dimension ref="A1:E158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:52:01</t>
+          <t>Última actualización: 13:10:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 140</t>
+          <t>Total filas: 153</t>
         </is>
       </c>
     </row>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1533,11 +1533,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>33</v>
+        <v>74</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -3323,12 +3323,12 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>13:14</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -3337,7 +3337,7 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3353,16 +3353,16 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,21 +3373,21 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>13:23</t>
+          <t>13:22</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,21 +3398,21 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:23</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>91</v>
+        <v>13</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,21 +3423,21 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:23</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,21 +3448,21 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>13:27</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,21 +3473,21 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>13:31</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>58</v>
+        <v>91</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,12 +3498,12 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>13:31</t>
+          <t>13:27</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -3512,7 +3512,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>81</v>
+        <v>54</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,12 +3523,12 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:31</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -3537,7 +3537,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,21 +3548,21 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>13:44</t>
+          <t>13:31</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3578,16 +3578,16 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>13:45</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,21 +3598,21 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>13:44</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>63</v>
+        <v>34</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3628,16 +3628,16 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>13:56</t>
+          <t>13:45</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,21 +3648,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>14:03</t>
+          <t>13:54</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>113</v>
+        <v>44</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3678,16 +3678,16 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>14:04</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,21 +3698,21 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>14:12</t>
+          <t>13:56</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>80</v>
+        <v>46</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,12 +3723,12 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>14:13</t>
+          <t>14:03</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -3737,7 +3737,7 @@
         </is>
       </c>
       <c r="D136" t="n">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,21 +3748,21 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:03</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>82</v>
+        <v>53</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3778,16 +3778,16 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:04</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3803,16 +3803,16 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>14:15</t>
+          <t>14:12</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,21 +3823,21 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:13</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>85</v>
+        <v>63</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3848,21 +3848,21 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:13</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>111</v>
+        <v>63</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3873,21 +3873,21 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>14:13</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,21 +3898,21 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>14:31</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>99</v>
+        <v>64</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3928,16 +3928,16 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>14:35</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>103</v>
+        <v>82</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3953,18 +3953,343 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>82</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>12:52:01</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>83</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>13:10:57</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>66</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>12:52:01</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>85</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>13:10:57</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>14:24</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>74</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>12:52:01</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>93</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>13:10:57</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>14:31</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>81</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>13:10:57</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>14:34</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>84</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>12:52:01</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>103</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>13:10:57</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>14:43</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>93</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>12:52:01</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
           <t>14:44</t>
         </is>
       </c>
-      <c r="C145" t="inlineStr">
+      <c r="C155" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D145" t="n">
+      <c r="D155" t="n">
         <v>112</v>
       </c>
-      <c r="E145" t="inlineStr">
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>13:10:57</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>104</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>13:10:57</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>15:03</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>113</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>13:10:57</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>114</v>
+      </c>
+      <c r="E158" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3981,7 +4306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3994,14 +4319,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:52:01</t>
+          <t>Última actualización: 13:10:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -4435,7 +4760,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -4449,7 +4774,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>58</v>
+        <v>21</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -4485,23 +4810,98 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>13:10:57</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>14:34</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>84</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>12:52:01</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>14:35</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D24" t="n">
+      <c r="D25" t="n">
         <v>103</v>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>13:10:57</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>104</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>13:10:57</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>114</v>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4518,7 +4918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4531,14 +4931,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:52:01</t>
+          <t>Última actualización: 13:10:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 23</t>
+          <t>Total filas: 24</t>
         </is>
       </c>
     </row>
@@ -5022,7 +5422,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -5036,7 +5436,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -5072,7 +5472,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -5086,7 +5486,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>76</v>
+        <v>39</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -5122,23 +5522,48 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>13:10:57</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>14:42</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>92</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>12:52:01</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>14:43</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D28" t="n">
+      <c r="D29" t="n">
         <v>111</v>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4660
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E158"/>
+  <dimension ref="A1:E165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:10:57</t>
+          <t>Última actualización: 13:43:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 153</t>
+          <t>Total filas: 160</t>
         </is>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>45</v>
+        <v>105</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>105</v>
+        <v>45</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>33</v>
+        <v>74</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>32</v>
+        <v>91</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>91</v>
+        <v>32</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>21</v>
+        <v>81</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>13:43:21</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3612,7 +3612,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3673,7 +3673,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>13:43:21</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -3687,7 +3687,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>63</v>
+        <v>12</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,7 +3698,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>13:43:21</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -3712,7 +3712,7 @@
         </is>
       </c>
       <c r="D135" t="n">
-        <v>46</v>
+        <v>13</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>13:43:21</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3787,7 +3787,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>72</v>
+        <v>21</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3798,21 +3798,21 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>13:43:21</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>14:12</t>
+          <t>14:05</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>80</v>
+        <v>22</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,21 +3823,21 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>13:43:21</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>14:13</t>
+          <t>14:11</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>63</v>
+        <v>28</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3848,21 +3848,21 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>14:13</t>
+          <t>14:12</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>63</v>
+        <v>80</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3883,11 +3883,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>100</v>
+        <v>63</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3903,16 +3903,16 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:13</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,21 +3923,21 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:13</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>82</v>
+        <v>100</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3958,11 +3958,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,21 +3973,21 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>13:43:21</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>14:15</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>83</v>
+        <v>31</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,21 +3998,21 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>13:43:21</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>66</v>
+        <v>31</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4028,7 +4028,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:15</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -4037,7 +4037,7 @@
         </is>
       </c>
       <c r="D148" t="n">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4053,16 +4053,16 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,21 +4073,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>13:43:21</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>93</v>
+        <v>34</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,21 +4098,21 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>13:43:21</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>14:31</t>
+          <t>14:24</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>81</v>
+        <v>41</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,21 +4123,21 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>14:34</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,21 +4148,21 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>13:43:21</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>14:35</t>
+          <t>14:31</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>103</v>
+        <v>48</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4178,16 +4178,16 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>14:43</t>
+          <t>14:34</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>93</v>
+        <v>84</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,21 +4198,21 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>13:43:21</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>14:44</t>
+          <t>14:35</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>112</v>
+        <v>52</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4228,16 +4228,16 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>14:54</t>
+          <t>14:43</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4248,21 +4248,21 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>13:43:21</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>15:03</t>
+          <t>14:44</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>113</v>
+        <v>61</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4278,18 +4278,193 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>104</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>13:43:21</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>72</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>13:10:57</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>15:03</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>113</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>13:43:21</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
           <t>15:04</t>
         </is>
       </c>
-      <c r="C158" t="inlineStr">
+      <c r="C161" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D158" t="n">
-        <v>114</v>
-      </c>
-      <c r="E158" t="inlineStr">
+      <c r="D161" t="n">
+        <v>81</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>13:43:21</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>15:09</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>86</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>13:43:21</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>92</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>13:43:21</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>15:24</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>101</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>13:43:21</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>112</v>
+      </c>
+      <c r="E165" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4306,7 +4481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4319,14 +4494,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:10:57</t>
+          <t>Última actualización: 13:43:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 24</t>
         </is>
       </c>
     </row>
@@ -4835,7 +5010,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>13:43:21</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -4849,7 +5024,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>103</v>
+        <v>52</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -4885,23 +5060,73 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>13:43:21</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>72</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>13:43:21</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
           <t>15:04</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D27" t="n">
-        <v>114</v>
-      </c>
-      <c r="E27" t="inlineStr">
+      <c r="D28" t="n">
+        <v>81</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>13:43:21</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>112</v>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4918,7 +5143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4931,14 +5156,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:10:57</t>
+          <t>Última actualización: 13:43:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 24</t>
+          <t>Total filas: 25</t>
         </is>
       </c>
     </row>
@@ -5497,7 +5722,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>13:43:21</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -5511,7 +5736,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>58</v>
+        <v>7</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -5547,7 +5772,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>13:43:21</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -5561,11 +5786,36 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>111</v>
+        <v>60</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>13:43:21</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>100</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4661
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E165"/>
+  <dimension ref="A1:E170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:43:21</t>
+          <t>Última actualización: 14:01:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 160</t>
+          <t>Total filas: 165</t>
         </is>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1533,11 +1533,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>59</v>
+        <v>12</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>10:46:10</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2633,11 +2633,11 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>12</v>
+        <v>59</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>21</v>
+        <v>81</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3723,12 +3723,12 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>14:03</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -3737,7 +3737,7 @@
         </is>
       </c>
       <c r="D136" t="n">
-        <v>113</v>
+        <v>1</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3773,21 +3773,21 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>13:43:21</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>14:04</t>
+          <t>14:03</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>21</v>
+        <v>113</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3798,21 +3798,21 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>13:43:21</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>14:05</t>
+          <t>14:04</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3828,16 +3828,16 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>14:11</t>
+          <t>14:05</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3848,12 +3848,12 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>14:12</t>
+          <t>14:11</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -3862,7 +3862,7 @@
         </is>
       </c>
       <c r="D141" t="n">
-        <v>80</v>
+        <v>10</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3873,21 +3873,21 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>14:13</t>
+          <t>14:12</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>63</v>
+        <v>80</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3953,16 +3953,16 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:13</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>13:43:21</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3987,7 +3987,7 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,7 +3998,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>13:43:21</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4008,11 +4008,11 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>31</v>
+        <v>64</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,21 +4023,21 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>14:15</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>83</v>
+        <v>13</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,12 +4048,12 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:15</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -4062,7 +4062,7 @@
         </is>
       </c>
       <c r="D149" t="n">
-        <v>66</v>
+        <v>83</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,12 +4073,12 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>13:43:21</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -4087,7 +4087,7 @@
         </is>
       </c>
       <c r="D150" t="n">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4103,16 +4103,16 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,12 +4123,12 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>14:24</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -4137,7 +4137,7 @@
         </is>
       </c>
       <c r="D152" t="n">
-        <v>93</v>
+        <v>23</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,21 +4148,21 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>13:43:21</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>14:31</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>48</v>
+        <v>93</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,21 +4173,21 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>14:34</t>
+          <t>14:31</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>84</v>
+        <v>30</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,12 +4198,12 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>13:43:21</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>14:35</t>
+          <t>14:34</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -4212,7 +4212,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>52</v>
+        <v>84</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,21 +4223,21 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>14:43</t>
+          <t>14:35</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>93</v>
+        <v>34</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4248,12 +4248,12 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>13:43:21</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>14:44</t>
+          <t>14:43</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -4262,7 +4262,7 @@
         </is>
       </c>
       <c r="D157" t="n">
-        <v>61</v>
+        <v>93</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,21 +4273,21 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>14:54</t>
+          <t>14:44</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>104</v>
+        <v>43</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,12 +4298,12 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>13:43:21</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>14:54</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -4312,7 +4312,7 @@
         </is>
       </c>
       <c r="D159" t="n">
-        <v>72</v>
+        <v>104</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,21 +4323,21 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>15:03</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>113</v>
+        <v>54</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,21 +4348,21 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>13:43:21</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>15:04</t>
+          <t>15:03</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>81</v>
+        <v>113</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,21 +4373,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>13:43:21</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>15:09</t>
+          <t>15:04</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>86</v>
+        <v>63</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,21 +4398,21 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>13:43:21</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:07</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4428,16 +4428,16 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:09</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,23 +4448,148 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>13:43:21</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>69</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>14:01:31</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>74</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>14:01:31</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>15:24</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>83</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>14:01:31</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
           <t>15:35</t>
         </is>
       </c>
-      <c r="C165" t="inlineStr">
+      <c r="C168" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D165" t="n">
-        <v>112</v>
-      </c>
-      <c r="E165" t="inlineStr">
+      <c r="D168" t="n">
+        <v>94</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>14:01:31</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>15:44</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>103</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>14:01:31</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>114</v>
+      </c>
+      <c r="E170" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4494,7 +4619,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:43:21</t>
+          <t>Última actualización: 14:01:31</t>
         </is>
       </c>
     </row>
@@ -5010,7 +5135,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>13:43:21</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -5024,7 +5149,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -5060,7 +5185,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>13:43:21</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -5074,7 +5199,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -5085,7 +5210,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>13:43:21</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -5099,7 +5224,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -5110,7 +5235,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>13:43:21</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -5124,7 +5249,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>112</v>
+        <v>94</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -5156,7 +5281,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:43:21</t>
+          <t>Última actualización: 14:01:31</t>
         </is>
       </c>
     </row>
@@ -5772,7 +5897,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>13:43:21</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -5786,7 +5911,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -5797,7 +5922,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>13:43:21</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -5811,7 +5936,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4662
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E170"/>
+  <dimension ref="A1:E180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:01:31</t>
+          <t>Última actualización: 14:28:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 165</t>
+          <t>Total filas: 175</t>
         </is>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>105</v>
+        <v>45</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>45</v>
+        <v>105</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>33</v>
+        <v>74</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>10:46:10</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>12</v>
+        <v>59</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2633,11 +2633,11 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>59</v>
+        <v>12</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>91</v>
+        <v>32</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>32</v>
+        <v>91</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>100</v>
+        <v>63</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3958,11 +3958,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>13</v>
+        <v>64</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,7 +3998,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4008,11 +4008,11 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>64</v>
+        <v>13</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4033,7 +4033,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -4173,21 +4173,21 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>14:31</t>
+          <t>14:29</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,21 +4198,21 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>14:34</t>
+          <t>14:31</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>84</v>
+        <v>3</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,12 +4223,12 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>14:35</t>
+          <t>14:34</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -4237,7 +4237,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>34</v>
+        <v>6</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4248,21 +4248,21 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>14:43</t>
+          <t>14:35</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>93</v>
+        <v>34</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,12 +4273,12 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>14:44</t>
+          <t>14:43</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -4287,7 +4287,7 @@
         </is>
       </c>
       <c r="D158" t="n">
-        <v>43</v>
+        <v>15</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,21 +4298,21 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>14:54</t>
+          <t>14:44</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>104</v>
+        <v>43</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,12 +4323,12 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>14:54</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -4337,7 +4337,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>54</v>
+        <v>26</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,21 +4348,21 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>15:03</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>113</v>
+        <v>54</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,21 +4373,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>15:04</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,21 +4398,21 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>15:07</t>
+          <t>15:03</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>66</v>
+        <v>113</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,21 +4423,21 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>13:43:21</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>15:09</t>
+          <t>15:04</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>86</v>
+        <v>36</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,21 +4448,21 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>15:10</t>
+          <t>15:06</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4478,16 +4478,16 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:07</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,21 +4498,21 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>13:43:21</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:09</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4528,16 +4528,16 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>15:35</t>
+          <t>15:10</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>94</v>
+        <v>69</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,21 +4548,21 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>15:44</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>103</v>
+        <v>47</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,23 +4573,273 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
+          <t>14:28:51</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>55</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
           <t>14:01:31</t>
         </is>
       </c>
-      <c r="B170" t="inlineStr">
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>15:24</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>83</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>14:28:51</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>66</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>14:01:31</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>94</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>14:28:51</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>15:44</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>76</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>14:28:51</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>15:51</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>83</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>14:28:51</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
         <is>
           <t>15:55</t>
         </is>
       </c>
-      <c r="C170" t="inlineStr">
+      <c r="C176" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D170" t="n">
-        <v>114</v>
-      </c>
-      <c r="E170" t="inlineStr">
+      <c r="D176" t="n">
+        <v>87</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>14:28:51</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>15:58</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>90</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>14:28:51</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>16:03</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>95</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>14:28:51</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>106</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>14:28:51</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>116</v>
+      </c>
+      <c r="E180" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4606,7 +4856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4619,14 +4869,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:01:31</t>
+          <t>Última actualización: 14:28:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 24</t>
+          <t>Total filas: 25</t>
         </is>
       </c>
     </row>
@@ -5110,7 +5360,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -5124,7 +5374,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>84</v>
+        <v>6</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -5160,7 +5410,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -5174,7 +5424,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>104</v>
+        <v>26</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -5210,7 +5460,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -5224,7 +5474,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>63</v>
+        <v>36</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -5235,23 +5485,48 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>14:28:51</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>66</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>14:01:31</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>15:35</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D29" t="n">
+      <c r="D30" t="n">
         <v>94</v>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5268,7 +5543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5281,14 +5556,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:01:31</t>
+          <t>Última actualización: 14:28:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 25</t>
+          <t>Total filas: 27</t>
         </is>
       </c>
     </row>
@@ -5872,7 +6147,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -5886,7 +6161,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>92</v>
+        <v>14</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -5922,25 +6197,75 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>14:28:51</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>15:22</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>54</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>14:01:31</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>15:23</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D30" t="n">
+      <c r="D31" t="n">
         <v>82</v>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>14:28:51</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>16:02</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>94</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4663
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E180"/>
+  <dimension ref="A1:E189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:28:51</t>
+          <t>Última actualización: 14:44:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 175</t>
+          <t>Total filas: 184</t>
         </is>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1533,11 +1533,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>32</v>
+        <v>91</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>91</v>
+        <v>32</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -3933,7 +3933,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>64</v>
+        <v>13</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,7 +3998,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4008,11 +4008,11 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>13</v>
+        <v>64</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4033,7 +4033,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>14:44:34</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4312,7 +4312,7 @@
         </is>
       </c>
       <c r="D159" t="n">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>14:44:34</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4362,7 +4362,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>54</v>
+        <v>11</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4398,12 +4398,12 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:44:34</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>15:03</t>
+          <t>15:02</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -4412,7 +4412,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>113</v>
+        <v>18</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,21 +4423,21 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>15:04</t>
+          <t>15:03</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>36</v>
+        <v>113</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,21 +4448,21 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>14:44:34</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>15:06</t>
+          <t>15:04</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4473,12 +4473,12 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>15:07</t>
+          <t>15:06</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -4487,7 +4487,7 @@
         </is>
       </c>
       <c r="D166" t="n">
-        <v>66</v>
+        <v>38</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,21 +4498,21 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>13:43:21</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>15:09</t>
+          <t>15:07</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>86</v>
+        <v>66</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,12 +4523,12 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>13:43:21</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>15:10</t>
+          <t>15:09</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -4537,7 +4537,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,21 +4548,21 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:10</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>47</v>
+        <v>69</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,21 +4573,21 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>14:44:34</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>15:23</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,12 +4598,12 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:23</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -4612,7 +4612,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>83</v>
+        <v>55</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,21 +4623,21 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>14:44:34</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>15:34</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>66</v>
+        <v>40</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,21 +4648,21 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>14:44:34</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>15:35</t>
+          <t>15:25</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>94</v>
+        <v>41</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4678,16 +4678,16 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>15:44</t>
+          <t>15:34</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,21 +4698,21 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>14:44:34</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>15:51</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>83</v>
+        <v>51</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,21 +4723,21 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>14:44:34</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>87</v>
+        <v>57</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,21 +4748,21 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>14:44:34</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>15:58</t>
+          <t>15:44</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4778,16 +4778,16 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>16:03</t>
+          <t>15:51</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,21 +4798,21 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>14:44:34</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>16:14</t>
+          <t>15:53</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>106</v>
+        <v>69</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,23 +4823,248 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
+          <t>14:44:34</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>71</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
           <t>14:28:51</t>
         </is>
       </c>
-      <c r="B180" t="inlineStr">
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>15:58</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>90</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>14:44:34</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>16:02</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>78</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>14:28:51</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>16:03</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>95</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>14:44:34</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>16:04</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>80</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>14:44:34</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>90</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>14:44:34</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>16:17</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>93</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>14:44:34</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
         <is>
           <t>16:24</t>
         </is>
       </c>
-      <c r="C180" t="inlineStr">
+      <c r="C187" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D180" t="n">
-        <v>116</v>
-      </c>
-      <c r="E180" t="inlineStr">
+      <c r="D187" t="n">
+        <v>100</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>14:44:34</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>16:34</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>110</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>14:44:34</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>111</v>
+      </c>
+      <c r="E189" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4869,7 +5094,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:28:51</t>
+          <t>Última actualización: 14:44:34</t>
         </is>
       </c>
     </row>
@@ -5435,7 +5660,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>14:44:34</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -5449,7 +5674,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>54</v>
+        <v>11</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -5460,7 +5685,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>14:44:34</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -5474,7 +5699,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -5510,7 +5735,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>14:44:34</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -5524,7 +5749,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>94</v>
+        <v>51</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -5543,7 +5768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5556,14 +5781,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:28:51</t>
+          <t>Última actualización: 14:44:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 27</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -6197,37 +6422,37 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>14:44:34</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>14:44</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>54</v>
+        <v>0</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>15:23</t>
+          <t>15:22</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -6236,7 +6461,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>82</v>
+        <v>54</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -6247,25 +6472,75 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>14:44:34</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>39</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>14:44:34</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
           <t>16:02</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D32" t="n">
-        <v>94</v>
-      </c>
-      <c r="E32" t="inlineStr">
+      <c r="D33" t="n">
+        <v>78</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>14:44:34</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>106</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4664
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E189"/>
+  <dimension ref="A1:E195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:44:34</t>
+          <t>Última actualización: 14:56:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 184</t>
+          <t>Total filas: 190</t>
         </is>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -3933,7 +3933,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -3998,7 +3998,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4008,11 +4008,11 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>64</v>
+        <v>13</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>13</v>
+        <v>64</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4373,21 +4373,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>14:56:45</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>15:01</t>
+          <t>14:56</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,12 +4398,12 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>14:44:34</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>15:02</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -4412,7 +4412,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,12 +4423,12 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:44:34</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>15:03</t>
+          <t>15:02</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -4437,7 +4437,7 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>113</v>
+        <v>18</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,21 +4448,21 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>14:44:34</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>15:04</t>
+          <t>15:03</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>20</v>
+        <v>113</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4473,21 +4473,21 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>14:56:45</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>15:06</t>
+          <t>15:04</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,21 +4498,21 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>14:56:45</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>15:07</t>
+          <t>15:04</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>66</v>
+        <v>8</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,21 +4523,21 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>13:43:21</t>
+          <t>14:56:45</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>15:09</t>
+          <t>15:06</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>86</v>
+        <v>10</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4553,16 +4553,16 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>15:10</t>
+          <t>15:07</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,21 +4573,21 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>14:44:34</t>
+          <t>13:43:21</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:09</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>31</v>
+        <v>86</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,21 +4598,21 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>15:23</t>
+          <t>15:10</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>55</v>
+        <v>69</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,21 +4623,21 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>14:44:34</t>
+          <t>14:56:45</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,21 +4648,21 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>14:44:34</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>15:25</t>
+          <t>15:23</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,21 +4673,21 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>14:56:45</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>15:34</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>66</v>
+        <v>28</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4703,16 +4703,16 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>15:35</t>
+          <t>15:25</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,21 +4723,21 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>14:44:34</t>
+          <t>14:56:45</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:28</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>57</v>
+        <v>32</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,21 +4748,21 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>14:44:34</t>
+          <t>14:56:45</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>15:44</t>
+          <t>15:34</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>60</v>
+        <v>38</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,21 +4773,21 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>14:44:34</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>15:51</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>83</v>
+        <v>51</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,21 +4798,21 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>14:44:34</t>
+          <t>14:56:45</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>15:53</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>69</v>
+        <v>45</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,21 +4823,21 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>14:44:34</t>
+          <t>14:56:45</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:44</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>71</v>
+        <v>48</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4853,16 +4853,16 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>15:58</t>
+          <t>15:51</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4878,16 +4878,16 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>16:02</t>
+          <t>15:53</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,21 +4898,21 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>14:56:45</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>16:03</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>95</v>
+        <v>59</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,21 +4923,21 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>14:44:34</t>
+          <t>14:56:45</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>16:04</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,21 +4948,21 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>14:44:34</t>
+          <t>14:56:45</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>16:14</t>
+          <t>15:58</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>90</v>
+        <v>62</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4978,16 +4978,16 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>16:17</t>
+          <t>16:02</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,21 +4998,21 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>14:44:34</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>16:03</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,21 +5023,21 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>14:44:34</t>
+          <t>14:56:45</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>16:34</t>
+          <t>16:04</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>110</v>
+        <v>68</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,23 +5048,173 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
+          <t>14:56:45</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>78</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
           <t>14:44:34</t>
         </is>
       </c>
-      <c r="B189" t="inlineStr">
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>16:17</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>93</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>14:56:45</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>88</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>14:56:45</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>16:34</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>98</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>14:56:45</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
         <is>
           <t>16:35</t>
         </is>
       </c>
-      <c r="C189" t="inlineStr">
+      <c r="C193" t="inlineStr">
         <is>
           <t>83_ALUAR</t>
         </is>
       </c>
-      <c r="D189" t="n">
-        <v>111</v>
-      </c>
-      <c r="E189" t="inlineStr">
+      <c r="D193" t="n">
+        <v>99</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>14:56:45</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>16:44</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>108</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>14:56:45</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>119</v>
+      </c>
+      <c r="E195" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5081,7 +5231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5094,14 +5244,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:44:34</t>
+          <t>Última actualización: 14:56:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 25</t>
+          <t>Total filas: 26</t>
         </is>
       </c>
     </row>
@@ -5685,21 +5835,21 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>14:44:34</t>
+          <t>14:56:45</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>15:04</t>
+          <t>14:56</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -5710,21 +5860,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>14:56:45</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>15:34</t>
+          <t>15:04</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>66</v>
+        <v>8</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -5735,23 +5885,48 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>14:56:45</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>38</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>14:44:34</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>15:35</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D30" t="n">
+      <c r="D31" t="n">
         <v>51</v>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5768,7 +5943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5781,14 +5956,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:44:34</t>
+          <t>Última actualización: 14:56:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -6447,7 +6622,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>14:56:45</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -6461,7 +6636,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>54</v>
+        <v>26</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -6497,7 +6672,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>14:44:34</t>
+          <t>14:56:45</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -6511,7 +6686,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -6522,23 +6697,48 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>14:56:45</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>16:29</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>93</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>14:44:34</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>16:30</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-40 Y 115</t>
         </is>
       </c>
-      <c r="D34" t="n">
+      <c r="D35" t="n">
         <v>106</v>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4665
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E195"/>
+  <dimension ref="A1:E204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:56:46</t>
+          <t>Última actualización: 15:17:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 190</t>
+          <t>Total filas: 199</t>
         </is>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>45</v>
+        <v>105</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>105</v>
+        <v>45</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1533,11 +1533,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>33</v>
+        <v>74</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>91</v>
+        <v>32</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>32</v>
+        <v>91</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>21</v>
+        <v>81</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3933,7 +3933,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3958,11 +3958,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>100</v>
+        <v>63</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>13</v>
+        <v>64</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -4008,7 +4008,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>64</v>
+        <v>13</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -4508,7 +4508,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -4648,12 +4648,12 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>15:23</t>
+          <t>15:19</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -4662,7 +4662,7 @@
         </is>
       </c>
       <c r="D173" t="n">
-        <v>55</v>
+        <v>2</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,12 +4673,12 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>14:56:45</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:23</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -4687,7 +4687,7 @@
         </is>
       </c>
       <c r="D174" t="n">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,21 +4698,21 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>14:44:34</t>
+          <t>14:56:45</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>15:25</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,12 +4723,12 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>14:56:45</t>
+          <t>14:44:34</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>15:28</t>
+          <t>15:25</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -4737,7 +4737,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4753,16 +4753,16 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>15:34</t>
+          <t>15:28</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,12 +4773,12 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>14:44:34</t>
+          <t>14:56:45</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>15:35</t>
+          <t>15:34</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -4787,7 +4787,7 @@
         </is>
       </c>
       <c r="D178" t="n">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,21 +4798,21 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>14:56:45</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,21 +4823,21 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>14:56:45</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>15:44</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,21 +4848,21 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>14:56:45</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>15:51</t>
+          <t>15:44</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>83</v>
+        <v>48</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,21 +4873,21 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>14:44:34</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>15:53</t>
+          <t>15:45</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>69</v>
+        <v>28</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,21 +4898,21 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>14:56:45</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:51</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>59</v>
+        <v>34</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,12 +4923,12 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>14:56:45</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:51</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -4937,7 +4937,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,21 +4948,21 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>14:56:45</t>
+          <t>14:44:34</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>15:58</t>
+          <t>15:53</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,21 +4973,21 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>14:44:34</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>16:02</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>78</v>
+        <v>38</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,21 +4998,21 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>14:56:45</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>16:03</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>95</v>
+        <v>60</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,21 +5023,21 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>14:56:45</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>16:04</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>68</v>
+        <v>40</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5053,16 +5053,16 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>16:14</t>
+          <t>15:58</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5078,16 +5078,16 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>16:17</t>
+          <t>16:02</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,21 +5098,21 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>14:56:45</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>16:03</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,21 +5123,21 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>14:56:45</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>16:34</t>
+          <t>16:04</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>98</v>
+        <v>47</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,21 +5148,21 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>14:56:45</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:14</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>99</v>
+        <v>57</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,21 +5173,21 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>14:56:45</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>16:44</t>
+          <t>16:16</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>108</v>
+        <v>59</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5198,23 +5198,248 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
+          <t>14:44:34</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>16:17</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>93</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
           <t>14:56:45</t>
         </is>
       </c>
-      <c r="B195" t="inlineStr">
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>88</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>15:17:10</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>16:25</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>68</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>15:17:10</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>16:34</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D198" t="n">
+        <v>77</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>15:17:10</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>78</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>15:17:10</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>16:41</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>84</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>15:17:10</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>16:44</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>87</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>15:17:10</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
         <is>
           <t>16:55</t>
         </is>
       </c>
-      <c r="C195" t="inlineStr">
+      <c r="C202" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D195" t="n">
-        <v>119</v>
-      </c>
-      <c r="E195" t="inlineStr">
+      <c r="D202" t="n">
+        <v>98</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>15:17:10</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>17:03</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>106</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>15:17:10</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D204" t="n">
+        <v>118</v>
+      </c>
+      <c r="E204" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5231,7 +5456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5244,14 +5469,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:56:46</t>
+          <t>Última actualización: 15:17:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 26</t>
+          <t>Total filas: 27</t>
         </is>
       </c>
     </row>
@@ -5910,7 +6135,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>14:44:34</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -5924,9 +6149,34 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>15:17:10</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>118</v>
+      </c>
+      <c r="E32" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5943,7 +6193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5956,14 +6206,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:56:46</t>
+          <t>Última actualización: 15:17:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 30</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -6647,7 +6897,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>14:44:34</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -6661,7 +6911,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -6697,48 +6947,98 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>14:56:45</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>16:29</t>
+          <t>16:03</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-40 Y 115</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>93</v>
+        <v>46</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>14:56:45</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>16:29</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>93</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>14:44:34</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>16:30</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-40 Y 115</t>
         </is>
       </c>
-      <c r="D35" t="n">
+      <c r="D36" t="n">
         <v>106</v>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>15:17:10</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>16:33</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>76</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4666
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E204"/>
+  <dimension ref="A1:E212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:17:10</t>
+          <t>Última actualización: 15:49:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 199</t>
+          <t>Total filas: 207</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>105</v>
+        <v>45</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>45</v>
+        <v>105</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>33</v>
+        <v>74</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>21</v>
+        <v>81</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>83</v>
+        <v>34</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,21 +4948,21 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>14:44:34</t>
+          <t>15:49:32</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>15:53</t>
+          <t>15:52</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>69</v>
+        <v>3</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,21 +4973,21 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>14:44:34</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:53</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,21 +4998,21 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>14:56:45</t>
+          <t>15:49:32</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>60</v>
+        <v>6</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,12 +5023,12 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>15:49:32</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -5037,7 +5037,7 @@
         </is>
       </c>
       <c r="D188" t="n">
-        <v>40</v>
+        <v>7</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,21 +5048,21 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>14:56:45</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>15:58</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,12 +5073,12 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>14:44:34</t>
+          <t>14:56:45</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>16:02</t>
+          <t>15:58</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -5087,7 +5087,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,21 +5098,21 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>14:44:34</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>16:03</t>
+          <t>16:02</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>95</v>
+        <v>78</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,12 +5123,12 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>16:04</t>
+          <t>16:03</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -5137,7 +5137,7 @@
         </is>
       </c>
       <c r="D192" t="n">
-        <v>47</v>
+        <v>95</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,21 +5148,21 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>15:49:32</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>16:14</t>
+          <t>16:04</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>57</v>
+        <v>15</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,21 +5173,21 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>15:49:32</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>16:16</t>
+          <t>16:14</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>59</v>
+        <v>25</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5198,12 +5198,12 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>14:44:34</t>
+          <t>15:49:32</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>16:17</t>
+          <t>16:16</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -5212,7 +5212,7 @@
         </is>
       </c>
       <c r="D195" t="n">
-        <v>93</v>
+        <v>27</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,21 +5223,21 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>14:56:45</t>
+          <t>14:44:34</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>16:17</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,12 +5248,12 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>15:49:32</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>16:25</t>
+          <t>16:24</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -5262,7 +5262,7 @@
         </is>
       </c>
       <c r="D197" t="n">
-        <v>68</v>
+        <v>35</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5278,16 +5278,16 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>16:34</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5298,21 +5298,21 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>15:49:32</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:34</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>78</v>
+        <v>45</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,21 +5323,21 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>15:49:32</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>16:41</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>84</v>
+        <v>46</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5353,16 +5353,16 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>16:44</t>
+          <t>16:41</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,21 +5373,21 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>15:49:32</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:44</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>98</v>
+        <v>55</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,21 +5398,21 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>15:49:32</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>17:03</t>
+          <t>16:51</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>106</v>
+        <v>62</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5423,23 +5423,223 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
+          <t>15:49:32</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D204" t="n">
+        <v>66</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
           <t>15:17:10</t>
         </is>
       </c>
-      <c r="B204" t="inlineStr">
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>17:03</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>106</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>15:49:32</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>17:04</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>75</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>15:49:32</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
         <is>
           <t>17:15</t>
         </is>
       </c>
-      <c r="C204" t="inlineStr">
+      <c r="C207" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D204" t="n">
-        <v>118</v>
-      </c>
-      <c r="E204" t="inlineStr">
+      <c r="D207" t="n">
+        <v>86</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>15:49:32</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>17:24</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>95</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>15:49:32</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>17:32</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>103</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>15:49:32</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>106</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>15:49:32</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D211" t="n">
+        <v>107</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>15:49:32</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>17:44</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>115</v>
+      </c>
+      <c r="E212" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5456,7 +5656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5469,14 +5669,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:17:10</t>
+          <t>Última actualización: 15:49:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 27</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -6160,7 +6360,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>15:49:32</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -6174,9 +6374,34 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>118</v>
+        <v>86</v>
       </c>
       <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>15:49:32</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>17:44</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>115</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6193,7 +6418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6206,14 +6431,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:17:10</t>
+          <t>Última actualización: 15:49:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 33</t>
         </is>
       </c>
     </row>
@@ -6947,7 +7172,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>15:49:32</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -6961,7 +7186,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -6997,7 +7222,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>14:44:34</t>
+          <t>15:49:32</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -7011,7 +7236,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>106</v>
+        <v>41</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -7041,6 +7266,31 @@
       <c r="E37" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>15:49:32</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>17:23</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>94</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4667
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E212"/>
+  <dimension ref="A1:E217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:49:32</t>
+          <t>Última actualización: 16:09:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 207</t>
+          <t>Total filas: 212</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>45</v>
+        <v>105</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>105</v>
+        <v>45</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1533,11 +1533,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>32</v>
+        <v>91</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>91</v>
+        <v>32</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>53</v>
+        <v>113</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3783,11 +3783,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>113</v>
+        <v>53</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -4508,7 +4508,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>83</v>
+        <v>34</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -5173,7 +5173,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -5187,7 +5187,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5198,7 +5198,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -5212,7 +5212,7 @@
         </is>
       </c>
       <c r="D195" t="n">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5262,7 +5262,7 @@
         </is>
       </c>
       <c r="D197" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5298,7 +5298,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -5312,7 +5312,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,7 +5323,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -5337,7 +5337,7 @@
         </is>
       </c>
       <c r="D200" t="n">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5362,7 +5362,7 @@
         </is>
       </c>
       <c r="D201" t="n">
-        <v>84</v>
+        <v>32</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,7 +5373,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -5387,7 +5387,7 @@
         </is>
       </c>
       <c r="D202" t="n">
-        <v>55</v>
+        <v>35</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,7 +5398,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5412,7 +5412,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>62</v>
+        <v>42</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5423,7 +5423,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -5437,7 +5437,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>66</v>
+        <v>46</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5473,7 +5473,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -5487,7 +5487,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5498,12 +5498,12 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>17:14</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -5512,7 +5512,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>86</v>
+        <v>65</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5528,16 +5528,16 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>17:24</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,21 +5548,21 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>103</v>
+        <v>75</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,21 +5573,21 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>106</v>
+        <v>83</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5603,16 +5603,16 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,23 +5623,148 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
+          <t>16:09:36</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>86</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>16:09:36</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>86</v>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
           <t>15:49:32</t>
         </is>
       </c>
-      <c r="B212" t="inlineStr">
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D214" t="n">
+        <v>107</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>16:09:36</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
         <is>
           <t>17:44</t>
         </is>
       </c>
-      <c r="C212" t="inlineStr">
+      <c r="C215" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D212" t="n">
-        <v>115</v>
-      </c>
-      <c r="E212" t="inlineStr">
+      <c r="D215" t="n">
+        <v>95</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>16:09:36</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D216" t="n">
+        <v>106</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>16:09:36</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>18:02</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D217" t="n">
+        <v>113</v>
+      </c>
+      <c r="E217" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5656,7 +5781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5669,14 +5794,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:49:32</t>
+          <t>Última actualización: 16:09:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -6360,12 +6485,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>17:14</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -6374,7 +6499,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>86</v>
+        <v>65</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -6390,18 +6515,68 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>86</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>16:09:36</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
           <t>17:44</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D33" t="n">
-        <v>115</v>
-      </c>
-      <c r="E33" t="inlineStr">
+      <c r="D34" t="n">
+        <v>95</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>16:09:36</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>106</v>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6418,7 +6593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6431,14 +6606,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:49:32</t>
+          <t>Última actualización: 16:09:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 33</t>
+          <t>Total filas: 34</t>
         </is>
       </c>
     </row>
@@ -7222,7 +7397,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -7236,7 +7411,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -7272,23 +7447,48 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>16:09:36</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>73</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>15:49:32</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>17:23</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D38" t="n">
+      <c r="D39" t="n">
         <v>94</v>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4668
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E217"/>
+  <dimension ref="A1:E225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:09:36</t>
+          <t>Última actualización: 16:31:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 212</t>
+          <t>Total filas: 220</t>
         </is>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>105</v>
+        <v>45</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>45</v>
+        <v>105</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>33</v>
+        <v>74</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>91</v>
+        <v>32</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>32</v>
+        <v>91</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>21</v>
+        <v>81</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>100</v>
+        <v>63</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3958,11 +3958,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>64</v>
+        <v>13</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -4008,7 +4008,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>13</v>
+        <v>64</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -4508,7 +4508,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>83</v>
+        <v>34</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -5298,21 +5298,21 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>16:34</t>
+          <t>16:31</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,21 +5323,21 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:34</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,21 +5348,21 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>16:41</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,21 +5373,21 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>16:44</t>
+          <t>16:41</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,21 +5398,21 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>16:51</t>
+          <t>16:44</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>42</v>
+        <v>13</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5423,21 +5423,21 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:51</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5448,21 +5448,21 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>17:03</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>106</v>
+        <v>24</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,12 +5473,12 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>17:04</t>
+          <t>17:03</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -5487,7 +5487,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>55</v>
+        <v>106</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5503,16 +5503,16 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>17:14</t>
+          <t>17:04</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,21 +5523,21 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>86</v>
+        <v>34</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5553,16 +5553,16 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>17:24</t>
+          <t>17:14</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,21 +5573,21 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>83</v>
+        <v>44</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,21 +5598,21 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>103</v>
+        <v>53</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,21 +5623,21 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:26</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,12 +5648,12 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>15:49:32</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -5662,7 +5662,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,12 +5673,12 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -5687,7 +5687,7 @@
         </is>
       </c>
       <c r="D214" t="n">
-        <v>107</v>
+        <v>61</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,21 +5698,21 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>17:44</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>95</v>
+        <v>64</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5728,16 +5728,16 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>106</v>
+        <v>86</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,23 +5748,223 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
+          <t>15:49:32</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D217" t="n">
+        <v>107</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>16:31:13</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>17:38</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D218" t="n">
+        <v>67</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
           <t>16:09:36</t>
         </is>
       </c>
-      <c r="B217" t="inlineStr">
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>17:44</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D219" t="n">
+        <v>95</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>16:31:13</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D220" t="n">
+        <v>74</v>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>16:31:13</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D221" t="n">
+        <v>84</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>16:09:36</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
         <is>
           <t>18:02</t>
         </is>
       </c>
-      <c r="C217" t="inlineStr">
+      <c r="C222" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D217" t="n">
+      <c r="D222" t="n">
         <v>113</v>
       </c>
-      <c r="E217" t="inlineStr">
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>16:31:13</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>18:04</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D223" t="n">
+        <v>93</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>16:31:13</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D224" t="n">
+        <v>104</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>16:31:13</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D225" t="n">
+        <v>114</v>
+      </c>
+      <c r="E225" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5781,7 +5981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5794,14 +5994,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:09:36</t>
+          <t>Última actualización: 16:31:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 30</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -6510,7 +6710,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -6524,7 +6724,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>86</v>
+        <v>44</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -6560,23 +6760,73 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>74</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>16:31:13</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
           <t>17:55</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D35" t="n">
-        <v>106</v>
-      </c>
-      <c r="E35" t="inlineStr">
+      <c r="D36" t="n">
+        <v>84</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>16:31:13</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>104</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6593,7 +6843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6606,14 +6856,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:09:36</t>
+          <t>Última actualización: 16:31:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 34</t>
+          <t>Total filas: 35</t>
         </is>
       </c>
     </row>
@@ -7447,48 +7697,73 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>17:22</t>
+          <t>16:41</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215B_LP-P MOR-40 Y 115</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>73</v>
+        <v>10</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>73</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>16:31:13</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
           <t>17:23</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D39" t="n">
-        <v>94</v>
-      </c>
-      <c r="E39" t="inlineStr">
+      <c r="D40" t="n">
+        <v>52</v>
+      </c>
+      <c r="E40" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4669
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E225"/>
+  <dimension ref="A1:E232"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:31:13</t>
+          <t>Última actualización: 16:49:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 220</t>
+          <t>Total filas: 227</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>45</v>
+        <v>105</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>105</v>
+        <v>45</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1533,11 +1533,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>32</v>
+        <v>91</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>91</v>
+        <v>32</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>113</v>
+        <v>53</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3783,11 +3783,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>53</v>
+        <v>113</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>13</v>
+        <v>64</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -4008,7 +4008,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>64</v>
+        <v>13</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -4508,7 +4508,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>83</v>
+        <v>34</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -5423,21 +5423,21 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>16:49:28</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>16:51</t>
+          <t>16:50</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5448,21 +5448,21 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>16:49:28</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:51</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,21 +5473,21 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>16:49:28</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>17:03</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>106</v>
+        <v>6</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5498,12 +5498,12 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>17:04</t>
+          <t>17:03</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -5512,7 +5512,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>55</v>
+        <v>106</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,12 +5523,12 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>16:49:28</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>17:05</t>
+          <t>17:04</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -5537,7 +5537,7 @@
         </is>
       </c>
       <c r="D208" t="n">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,21 +5548,21 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>17:14</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>65</v>
+        <v>34</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,12 +5573,12 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>17:14</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -5587,7 +5587,7 @@
         </is>
       </c>
       <c r="D210" t="n">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,21 +5598,21 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>16:49:28</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>17:24</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,21 +5623,21 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>16:49:28</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>17:26</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>55</v>
+        <v>35</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,21 +5648,21 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>17:26</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>103</v>
+        <v>55</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,21 +5673,21 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>16:49:28</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5703,16 +5703,16 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,12 +5723,12 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>15:49:32</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -5737,7 +5737,7 @@
         </is>
       </c>
       <c r="D216" t="n">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,21 +5748,21 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>107</v>
+        <v>86</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5773,21 +5773,21 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>16:49:28</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>67</v>
+        <v>46</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,21 +5798,21 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>16:49:28</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>17:44</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>95</v>
+        <v>47</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5828,16 +5828,16 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:38</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5848,21 +5848,21 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>16:49:28</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:44</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>84</v>
+        <v>55</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5873,21 +5873,21 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>18:02</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>113</v>
+        <v>74</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,21 +5898,21 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>16:49:28</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>18:04</t>
+          <t>17:55</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>93</v>
+        <v>66</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,21 +5923,21 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>18:15</t>
+          <t>18:02</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5948,23 +5948,198 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
+          <t>16:49:28</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>18:04</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D225" t="n">
+        <v>75</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>16:49:28</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>86</v>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>16:49:28</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>18:21</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D227" t="n">
+        <v>92</v>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>16:49:28</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>95</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
           <t>16:31:13</t>
         </is>
       </c>
-      <c r="B225" t="inlineStr">
+      <c r="B229" t="inlineStr">
         <is>
           <t>18:25</t>
         </is>
       </c>
-      <c r="C225" t="inlineStr">
+      <c r="C229" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D225" t="n">
+      <c r="D229" t="n">
         <v>114</v>
       </c>
-      <c r="E225" t="inlineStr">
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>16:49:28</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>18:34</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>105</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>16:49:28</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D231" t="n">
+        <v>107</v>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>16:49:28</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>18:44</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D232" t="n">
+        <v>115</v>
+      </c>
+      <c r="E232" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5994,7 +6169,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:31:13</t>
+          <t>Última actualización: 16:49:28</t>
         </is>
       </c>
     </row>
@@ -6710,7 +6885,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>16:49:28</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -6724,7 +6899,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -6735,7 +6910,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>16:49:28</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -6749,7 +6924,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>95</v>
+        <v>55</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -6785,7 +6960,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>16:49:28</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -6799,7 +6974,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -6810,7 +6985,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>16:49:28</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6824,7 +6999,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>104</v>
+        <v>86</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -6843,7 +7018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6856,14 +7031,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:31:13</t>
+          <t>Última actualización: 16:49:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 35</t>
+          <t>Total filas: 36</t>
         </is>
       </c>
     </row>
@@ -7747,7 +7922,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>16:49:28</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -7761,9 +7936,34 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="E40" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>16:49:28</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>116</v>
+      </c>
+      <c r="E41" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4670
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E232"/>
+  <dimension ref="A1:E234"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:49:28</t>
+          <t>Última actualización: 16:59:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 227</t>
+          <t>Total filas: 229</t>
         </is>
       </c>
     </row>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1533,11 +1533,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>33</v>
+        <v>74</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>21</v>
+        <v>81</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>53</v>
+        <v>113</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3783,11 +3783,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>113</v>
+        <v>53</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3958,11 +3958,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>100</v>
+        <v>63</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>64</v>
+        <v>13</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,7 +3998,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4008,11 +4008,11 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>13</v>
+        <v>64</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4033,7 +4033,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>83</v>
+        <v>34</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -5498,21 +5498,21 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>17:03</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>106</v>
+        <v>1</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,12 +5523,12 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>16:49:28</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>17:04</t>
+          <t>17:03</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -5537,7 +5537,7 @@
         </is>
       </c>
       <c r="D208" t="n">
-        <v>15</v>
+        <v>106</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,12 +5548,12 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>17:05</t>
+          <t>17:04</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -5562,7 +5562,7 @@
         </is>
       </c>
       <c r="D209" t="n">
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,21 +5573,21 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>17:14</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>65</v>
+        <v>34</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,12 +5598,12 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>16:49:28</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>17:14</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -5612,7 +5612,7 @@
         </is>
       </c>
       <c r="D211" t="n">
-        <v>26</v>
+        <v>65</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,21 +5623,21 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>16:49:28</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>17:24</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,21 +5648,21 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>17:26</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,21 +5673,21 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>16:49:28</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>17:31</t>
+          <t>17:26</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,21 +5698,21 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>61</v>
+        <v>32</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>103</v>
+        <v>61</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,12 +5748,12 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>15:49:32</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -5762,7 +5762,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5773,7 +5773,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>16:49:28</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -5783,11 +5783,11 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>46</v>
+        <v>86</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,21 +5798,21 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>16:49:28</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,21 +5823,21 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>67</v>
+        <v>37</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5848,21 +5848,21 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>16:49:28</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>17:44</t>
+          <t>17:38</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5873,12 +5873,12 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:44</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -5887,7 +5887,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>74</v>
+        <v>45</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,21 +5898,21 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>16:49:28</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,21 +5923,21 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>18:02</t>
+          <t>17:55</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>113</v>
+        <v>56</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5948,12 +5948,12 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>16:49:28</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>18:04</t>
+          <t>18:02</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="D225" t="n">
-        <v>75</v>
+        <v>113</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,21 +5973,21 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>16:49:28</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>18:15</t>
+          <t>18:04</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>86</v>
+        <v>65</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,21 +5998,21 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>16:49:28</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>18:21</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,21 +6023,21 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>16:49:28</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:21</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,12 +6048,12 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -6062,7 +6062,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>114</v>
+        <v>85</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6073,21 +6073,21 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>16:49:28</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>18:34</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,21 +6098,21 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>16:49:28</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:34</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,23 +6123,73 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>16:49:28</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D232" t="n">
+        <v>97</v>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>16:59:32</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
           <t>18:44</t>
         </is>
       </c>
-      <c r="C232" t="inlineStr">
+      <c r="C233" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D232" t="n">
+      <c r="D233" t="n">
+        <v>105</v>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>16:59:32</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>18:54</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D234" t="n">
         <v>115</v>
       </c>
-      <c r="E232" t="inlineStr">
+      <c r="E234" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6169,7 +6219,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:49:28</t>
+          <t>Última actualización: 16:59:32</t>
         </is>
       </c>
     </row>
@@ -6885,7 +6935,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>16:49:28</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -6899,7 +6949,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -6910,7 +6960,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>16:49:28</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -6924,7 +6974,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -6960,7 +7010,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>16:49:28</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -6974,7 +7024,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -6985,7 +7035,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>16:49:28</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6999,7 +7049,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -7031,7 +7081,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:49:28</t>
+          <t>Última actualización: 16:59:32</t>
         </is>
       </c>
     </row>
@@ -7922,7 +7972,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>16:49:28</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -7936,7 +7986,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -7947,7 +7997,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>16:49:28</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -7961,7 +8011,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4671
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E234"/>
+  <dimension ref="A1:E239"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:59:32</t>
+          <t>Última actualización: 17:21:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 229</t>
+          <t>Total filas: 234</t>
         </is>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1533,11 +1533,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>33</v>
+        <v>74</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>91</v>
+        <v>32</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>32</v>
+        <v>91</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>100</v>
+        <v>63</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3958,11 +3958,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3998,7 +3998,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4008,11 +4008,11 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>64</v>
+        <v>13</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>13</v>
+        <v>64</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -5648,21 +5648,21 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>17:24</t>
+          <t>17:22</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,21 +5673,21 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>17:26</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>27</v>
+        <v>3</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5703,16 +5703,16 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>17:31</t>
+          <t>17:26</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,21 +5723,21 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>61</v>
+        <v>10</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>103</v>
+        <v>61</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5773,12 +5773,12 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>15:49:32</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -5787,7 +5787,7 @@
         </is>
       </c>
       <c r="D218" t="n">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,7 +5798,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -5812,7 +5812,7 @@
         </is>
       </c>
       <c r="D219" t="n">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,21 +5823,21 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>37</v>
+        <v>86</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5848,21 +5848,21 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>67</v>
+        <v>15</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5873,21 +5873,21 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>17:44</t>
+          <t>17:38</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>45</v>
+        <v>67</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,12 +5898,12 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:44</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -5912,7 +5912,7 @@
         </is>
       </c>
       <c r="D223" t="n">
-        <v>74</v>
+        <v>23</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,21 +5923,21 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5948,21 +5948,21 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>18:02</t>
+          <t>17:55</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>113</v>
+        <v>34</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,12 +5973,12 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>18:04</t>
+          <t>18:02</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -5987,7 +5987,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>65</v>
+        <v>113</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,21 +5998,21 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>18:15</t>
+          <t>18:04</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>76</v>
+        <v>43</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,21 +6023,21 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>18:21</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>82</v>
+        <v>54</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6053,16 +6053,16 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:21</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6073,12 +6073,12 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -6087,7 +6087,7 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>114</v>
+        <v>63</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,21 +6098,21 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>18:34</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>95</v>
+        <v>114</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,21 +6123,21 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:34</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>97</v>
+        <v>73</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,21 +6148,21 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>18:44</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>105</v>
+        <v>75</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,23 +6173,148 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
+          <t>18:44</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D234" t="n">
+        <v>83</v>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>17:21:32</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
           <t>18:54</t>
         </is>
       </c>
-      <c r="C234" t="inlineStr">
+      <c r="C235" t="inlineStr">
         <is>
           <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
-      <c r="D234" t="n">
+      <c r="D235" t="n">
+        <v>93</v>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>17:21:32</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D236" t="n">
+        <v>99</v>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>17:21:32</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>19:11</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D237" t="n">
+        <v>110</v>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>17:21:32</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D238" t="n">
         <v>115</v>
       </c>
-      <c r="E234" t="inlineStr">
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>17:21:32</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D239" t="n">
+        <v>115</v>
+      </c>
+      <c r="E239" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6206,7 +6331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6219,14 +6344,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:59:32</t>
+          <t>Última actualización: 17:21:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 33</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6560,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -6445,11 +6570,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>105</v>
+        <v>45</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -6460,7 +6585,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -6470,11 +6595,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>45</v>
+        <v>105</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -6960,7 +7085,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -6974,7 +7099,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -7010,7 +7135,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -7024,7 +7149,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -7035,7 +7160,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -7049,9 +7174,34 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>76</v>
+        <v>54</v>
       </c>
       <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>17:21:32</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>99</v>
+      </c>
+      <c r="E38" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7068,7 +7218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7081,14 +7231,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:59:32</t>
+          <t>Última actualización: 17:21:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 36</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -7972,7 +8122,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -7986,7 +8136,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -7997,7 +8147,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -8011,11 +8161,36 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>106</v>
+        <v>84</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>17:21:32</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>114</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4672
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E239"/>
+  <dimension ref="A1:E243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:21:32</t>
+          <t>Última actualización: 17:44:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 234</t>
+          <t>Total filas: 238</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>105</v>
+        <v>45</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>45</v>
+        <v>105</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1533,11 +1533,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>32</v>
+        <v>91</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>91</v>
+        <v>32</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>21</v>
+        <v>81</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3958,11 +3958,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>100</v>
+        <v>63</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>13</v>
+        <v>64</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -4008,7 +4008,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>64</v>
+        <v>13</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -4508,7 +4508,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>15:49:32</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>61</v>
+        <v>103</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5773,7 +5773,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -5783,11 +5783,11 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>103</v>
+        <v>61</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5898,7 +5898,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5908,11 +5908,11 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,12 +5923,12 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:44</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -5937,7 +5937,7 @@
         </is>
       </c>
       <c r="D224" t="n">
-        <v>74</v>
+        <v>23</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5948,21 +5948,21 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,21 +5973,21 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>18:02</t>
+          <t>17:55</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>113</v>
+        <v>11</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,21 +5998,21 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>18:04</t>
+          <t>18:01</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,21 +6023,21 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>18:15</t>
+          <t>18:02</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>54</v>
+        <v>113</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,21 +6048,21 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>18:21</t>
+          <t>18:04</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>82</v>
+        <v>20</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6073,21 +6073,21 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>63</v>
+        <v>31</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,21 +6098,21 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:21</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>114</v>
+        <v>37</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,21 +6123,21 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>18:34</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>73</v>
+        <v>40</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,21 +6148,21 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,21 +6173,21 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>18:44</t>
+          <t>18:34</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>83</v>
+        <v>50</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6203,16 +6203,16 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>18:54</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,21 +6223,21 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:44</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>99</v>
+        <v>60</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6248,21 +6248,21 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>19:11</t>
+          <t>18:54</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>110</v>
+        <v>70</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -6273,21 +6273,21 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>115</v>
+        <v>76</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -6298,23 +6298,123 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
+          <t>19:11</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D239" t="n">
+        <v>87</v>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>17:44:31</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
           <t>19:16</t>
         </is>
       </c>
-      <c r="C239" t="inlineStr">
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D240" t="n">
+        <v>92</v>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>17:44:31</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D239" t="n">
-        <v>115</v>
-      </c>
-      <c r="E239" t="inlineStr">
+      <c r="D241" t="n">
+        <v>92</v>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>17:44:31</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D242" t="n">
+        <v>100</v>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>17:44:31</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>19:26</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D243" t="n">
+        <v>102</v>
+      </c>
+      <c r="E243" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6331,7 +6431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6344,14 +6444,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:21:32</t>
+          <t>Última actualización: 17:44:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 33</t>
+          <t>Total filas: 34</t>
         </is>
       </c>
     </row>
@@ -7110,7 +7210,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -7124,7 +7224,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>74</v>
+        <v>1</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -7135,7 +7235,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -7149,7 +7249,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -7160,7 +7260,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -7174,7 +7274,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>54</v>
+        <v>31</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -7185,7 +7285,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -7199,9 +7299,34 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>99</v>
+        <v>76</v>
       </c>
       <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>17:44:31</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>19:26</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>102</v>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7231,7 +7356,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:21:32</t>
+          <t>Última actualización: 17:44:31</t>
         </is>
       </c>
     </row>
@@ -8147,7 +8272,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -8161,7 +8286,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>84</v>
+        <v>61</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -8172,7 +8297,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -8186,7 +8311,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>114</v>
+        <v>91</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4673
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E243"/>
+  <dimension ref="A1:E251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:44:31</t>
+          <t>Última actualización: 17:58:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 238</t>
+          <t>Total filas: 246</t>
         </is>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>21</v>
+        <v>81</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>113</v>
+        <v>53</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3783,11 +3783,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>53</v>
+        <v>113</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>100</v>
+        <v>63</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3958,7 +3958,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>83</v>
+        <v>34</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -5898,7 +5898,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5908,11 +5908,11 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,7 +5923,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -5933,11 +5933,11 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5998,21 +5998,21 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>18:01</t>
+          <t>17:59</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,12 +6023,12 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>18:02</t>
+          <t>18:01</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -6037,7 +6037,7 @@
         </is>
       </c>
       <c r="D228" t="n">
-        <v>113</v>
+        <v>3</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6053,16 +6053,16 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>18:04</t>
+          <t>18:01</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6073,21 +6073,21 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>18:15</t>
+          <t>18:02</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>31</v>
+        <v>113</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6103,16 +6103,16 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>18:21</t>
+          <t>18:04</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,21 +6123,21 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:14</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,21 +6148,21 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>114</v>
+        <v>31</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,21 +6173,21 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>18:34</t>
+          <t>18:21</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,21 +6198,21 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>75</v>
+        <v>26</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,21 +6223,21 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>18:44</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6248,21 +6248,21 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>18:54</t>
+          <t>18:34</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>70</v>
+        <v>36</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -6273,21 +6273,21 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -6298,21 +6298,21 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>19:11</t>
+          <t>18:44</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>87</v>
+        <v>46</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,21 +6323,21 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>18:54</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>92</v>
+        <v>56</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6348,21 +6348,21 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>18:59</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>92</v>
+        <v>61</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6378,16 +6378,16 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>100</v>
+        <v>76</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6403,18 +6403,218 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
+          <t>19:11</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D243" t="n">
+        <v>87</v>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>17:58:44</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D244" t="n">
+        <v>77</v>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>17:58:44</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D245" t="n">
+        <v>78</v>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>17:58:44</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D246" t="n">
+        <v>78</v>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>17:58:44</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D247" t="n">
+        <v>86</v>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>17:44:31</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
           <t>19:26</t>
         </is>
       </c>
-      <c r="C243" t="inlineStr">
+      <c r="C248" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D243" t="n">
+      <c r="D248" t="n">
         <v>102</v>
       </c>
-      <c r="E243" t="inlineStr">
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>17:58:44</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D249" t="n">
+        <v>92</v>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>17:58:44</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>19:49</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D250" t="n">
+        <v>111</v>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>17:58:44</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D251" t="n">
+        <v>112</v>
+      </c>
+      <c r="E251" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6431,7 +6631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6444,14 +6644,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:44:31</t>
+          <t>Última actualización: 17:58:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 34</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -6620,7 +6820,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -6645,7 +6845,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -6660,7 +6860,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -6670,11 +6870,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>45</v>
+        <v>105</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -6685,7 +6885,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -6695,11 +6895,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>105</v>
+        <v>45</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -7260,12 +7460,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>18:15</t>
+          <t>18:14</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -7274,7 +7474,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -7290,16 +7490,16 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>76</v>
+        <v>31</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -7310,23 +7510,98 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>17:58:44</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>18:59</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>61</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>17:44:31</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>76</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>17:44:31</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
         <is>
           <t>19:26</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D39" t="n">
+      <c r="D41" t="n">
         <v>102</v>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>17:58:44</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>92</v>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7343,7 +7618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7356,14 +7631,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:44:31</t>
+          <t>Última actualización: 17:58:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 40</t>
         </is>
       </c>
     </row>
@@ -8272,12 +8547,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>18:45</t>
+          <t>18:44</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -8286,7 +8561,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -8302,20 +8577,95 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>61</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>17:58:44</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>19:14</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>76</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>17:44:31</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
           <t>19:15</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D42" t="n">
+      <c r="D44" t="n">
         <v>91</v>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E44" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>17:58:44</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>19:46</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>108</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4674
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E251"/>
+  <dimension ref="A1:E257"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:58:44</t>
+          <t>Última actualización: 18:18:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 246</t>
+          <t>Total filas: 252</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>45</v>
+        <v>105</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>105</v>
+        <v>45</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1533,11 +1533,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>33</v>
+        <v>74</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>59</v>
+        <v>12</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>10:46:10</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2633,11 +2633,11 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>12</v>
+        <v>59</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>91</v>
+        <v>32</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>32</v>
+        <v>91</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>21</v>
+        <v>81</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3933,7 +3933,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -3958,7 +3958,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>64</v>
+        <v>13</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,7 +3998,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4008,11 +4008,11 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>13</v>
+        <v>64</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>83</v>
+        <v>34</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>103</v>
+        <v>61</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5773,7 +5773,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>15:49:32</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -5783,11 +5783,11 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>61</v>
+        <v>103</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,7 +5798,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -5808,11 +5808,11 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>14</v>
+        <v>86</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,7 +5823,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -5833,11 +5833,11 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>86</v>
+        <v>14</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -6023,7 +6023,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>17:58:44</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -6033,11 +6033,11 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,7 +6048,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -6058,11 +6058,11 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6173,21 +6173,21 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>17:58:44</t>
+          <t>18:18:08</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>18:21</t>
+          <t>18:19</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6203,16 +6203,16 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:21</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,12 +6223,12 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -6237,7 +6237,7 @@
         </is>
       </c>
       <c r="D236" t="n">
-        <v>114</v>
+        <v>26</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6248,21 +6248,21 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>17:58:44</t>
+          <t>18:18:08</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>18:34</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>36</v>
+        <v>7</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -6273,21 +6273,21 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>17:58:44</t>
+          <t>18:18:08</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>38</v>
+        <v>7</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -6298,21 +6298,21 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>17:58:44</t>
+          <t>18:18:08</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>18:44</t>
+          <t>18:34</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,21 +6323,21 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>17:58:44</t>
+          <t>18:18:08</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>18:54</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>56</v>
+        <v>18</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6348,21 +6348,21 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>17:58:44</t>
+          <t>18:18:08</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>18:59</t>
+          <t>18:44</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>61</v>
+        <v>26</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,21 +6373,21 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>18:18:08</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:54</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>76</v>
+        <v>36</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6398,21 +6398,21 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>19:11</t>
+          <t>18:59</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D243" t="n">
-        <v>87</v>
+        <v>61</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -6423,21 +6423,21 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>17:58:44</t>
+          <t>18:18:08</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>19:15</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>77</v>
+        <v>42</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6448,21 +6448,21 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>17:58:44</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:11</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6478,16 +6478,16 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:15</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6498,21 +6498,21 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>17:58:44</t>
+          <t>18:18:08</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>86</v>
+        <v>58</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6523,21 +6523,21 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>18:18:08</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>19:26</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>102</v>
+        <v>58</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6553,16 +6553,16 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -6573,21 +6573,21 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>17:58:44</t>
+          <t>18:18:08</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>19:49</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>111</v>
+        <v>59</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6598,23 +6598,173 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
+          <t>18:18:08</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D251" t="n">
+        <v>66</v>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>17:44:31</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>19:26</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D252" t="n">
+        <v>102</v>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>18:18:08</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>19:27</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D253" t="n">
+        <v>69</v>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
           <t>17:58:44</t>
         </is>
       </c>
-      <c r="B251" t="inlineStr">
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D254" t="n">
+        <v>92</v>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>18:18:08</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>19:49</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D255" t="n">
+        <v>91</v>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>18:18:08</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
         <is>
           <t>19:50</t>
         </is>
       </c>
-      <c r="C251" t="inlineStr">
+      <c r="C256" t="inlineStr">
         <is>
           <t>81_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D251" t="n">
-        <v>112</v>
-      </c>
-      <c r="E251" t="inlineStr">
+      <c r="D256" t="n">
+        <v>92</v>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>18:18:08</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D257" t="n">
+        <v>117</v>
+      </c>
+      <c r="E257" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6631,7 +6781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6644,14 +6794,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:58:44</t>
+          <t>Última actualización: 18:18:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 39</t>
         </is>
       </c>
     </row>
@@ -6820,7 +6970,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -6845,7 +6995,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -7535,7 +7685,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>18:18:08</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -7549,7 +7699,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>76</v>
+        <v>42</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -7585,23 +7735,73 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>18:18:08</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>19:27</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>69</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>17:58:44</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D42" t="n">
+      <c r="D43" t="n">
         <v>92</v>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>18:18:08</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>117</v>
+      </c>
+      <c r="E44" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7618,7 +7818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7631,14 +7831,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:58:44</t>
+          <t>Última actualización: 18:18:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 40</t>
+          <t>Total filas: 41</t>
         </is>
       </c>
     </row>
@@ -8572,7 +8772,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>18:18:08</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -8586,7 +8786,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>61</v>
+        <v>27</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -8622,7 +8822,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>18:18:08</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -8636,7 +8836,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>91</v>
+        <v>57</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -8664,6 +8864,31 @@
         <v>108</v>
       </c>
       <c r="E45" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>18:18:08</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>19:47</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>89</v>
+      </c>
+      <c r="E46" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4675
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E257"/>
+  <dimension ref="A1:E261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:18:08</t>
+          <t>Última actualización: 18:38:18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 252</t>
+          <t>Total filas: 256</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>105</v>
+        <v>45</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>45</v>
+        <v>105</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1533,11 +1533,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>10:46:10</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>12</v>
+        <v>59</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2633,11 +2633,11 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>59</v>
+        <v>12</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -3998,7 +3998,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4008,11 +4008,11 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>64</v>
+        <v>13</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>13</v>
+        <v>64</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -4508,7 +4508,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>83</v>
+        <v>34</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>15:49:32</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>61</v>
+        <v>103</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5773,7 +5773,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -5783,11 +5783,11 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>103</v>
+        <v>61</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,7 +5798,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -5808,11 +5808,11 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>86</v>
+        <v>14</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,7 +5823,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -5833,11 +5833,11 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>14</v>
+        <v>86</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -6023,7 +6023,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -6033,11 +6033,11 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,7 +6048,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>17:58:44</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -6058,11 +6058,11 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6348,21 +6348,21 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>18:18:08</t>
+          <t>18:38:18</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>18:44</t>
+          <t>18:38</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,21 +6373,21 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>18:18:08</t>
+          <t>18:38:18</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>18:54</t>
+          <t>18:44</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>36</v>
+        <v>6</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6398,21 +6398,21 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>17:58:44</t>
+          <t>18:38:18</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>18:59</t>
+          <t>18:54</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D243" t="n">
-        <v>61</v>
+        <v>16</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -6423,12 +6423,12 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>18:18:08</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:59</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -6437,7 +6437,7 @@
         </is>
       </c>
       <c r="D244" t="n">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6448,21 +6448,21 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>18:38:18</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>19:11</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>87</v>
+        <v>22</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6473,12 +6473,12 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>17:58:44</t>
+          <t>18:38:18</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>19:15</t>
+          <t>19:11</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -6487,7 +6487,7 @@
         </is>
       </c>
       <c r="D246" t="n">
-        <v>77</v>
+        <v>33</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6498,12 +6498,12 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>18:18:08</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:15</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -6512,7 +6512,7 @@
         </is>
       </c>
       <c r="D247" t="n">
-        <v>58</v>
+        <v>77</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6523,7 +6523,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>18:18:08</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -6533,11 +6533,11 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6548,7 +6548,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>17:58:44</t>
+          <t>18:38:18</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -6558,11 +6558,11 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>78</v>
+        <v>38</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -6578,16 +6578,16 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6598,21 +6598,21 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>18:18:08</t>
+          <t>18:38:18</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>66</v>
+        <v>39</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -6623,21 +6623,21 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>18:38:18</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>19:26</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>102</v>
+        <v>46</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,12 +6648,12 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>18:18:08</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>19:27</t>
+          <t>19:26</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
@@ -6662,7 +6662,7 @@
         </is>
       </c>
       <c r="D253" t="n">
-        <v>69</v>
+        <v>102</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6673,12 +6673,12 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>17:58:44</t>
+          <t>18:18:08</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>19:27</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
@@ -6687,7 +6687,7 @@
         </is>
       </c>
       <c r="D254" t="n">
-        <v>92</v>
+        <v>69</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -6698,21 +6698,21 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>18:18:08</t>
+          <t>18:38:18</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>19:49</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>91</v>
+        <v>52</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6723,21 +6723,21 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>18:18:08</t>
+          <t>18:38:18</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>19:50</t>
+          <t>19:49</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>92</v>
+        <v>71</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6748,23 +6748,123 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>18:18:08</t>
+          <t>18:38:18</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D257" t="n">
+        <v>72</v>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>18:38:18</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>20:01</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D258" t="n">
+        <v>83</v>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>18:38:18</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>20:07</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D259" t="n">
+        <v>89</v>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>18:38:18</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
           <t>20:15</t>
         </is>
       </c>
-      <c r="C257" t="inlineStr">
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D260" t="n">
+        <v>97</v>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>18:38:18</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D257" t="n">
-        <v>117</v>
-      </c>
-      <c r="E257" t="inlineStr">
+      <c r="D261" t="n">
+        <v>97</v>
+      </c>
+      <c r="E261" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6794,7 +6894,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:18:08</t>
+          <t>Última actualización: 18:38:18</t>
         </is>
       </c>
     </row>
@@ -6970,7 +7070,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -6995,7 +7095,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -7685,7 +7785,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>18:18:08</t>
+          <t>18:38:18</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -7699,7 +7799,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -7760,7 +7860,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>17:58:44</t>
+          <t>18:38:18</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -7774,7 +7874,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>92</v>
+        <v>52</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -7785,7 +7885,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>18:18:08</t>
+          <t>18:38:18</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -7799,7 +7899,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>117</v>
+        <v>97</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -7831,7 +7931,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:18:08</t>
+          <t>Última actualización: 18:38:18</t>
         </is>
       </c>
     </row>
@@ -8772,7 +8872,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>18:18:08</t>
+          <t>18:38:18</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -8786,7 +8886,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -8822,7 +8922,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>18:18:08</t>
+          <t>18:38:18</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -8836,7 +8936,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -8872,7 +8972,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>18:18:08</t>
+          <t>18:38:18</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -8886,7 +8986,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>89</v>
+        <v>69</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4676
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E261"/>
+  <dimension ref="A1:E266"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:38:18</t>
+          <t>Última actualización: 18:53:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 256</t>
+          <t>Total filas: 261</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>32</v>
+        <v>91</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>91</v>
+        <v>32</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>21</v>
+        <v>81</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>100</v>
+        <v>63</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3958,11 +3958,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3983,7 +3983,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -4008,7 +4008,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -5798,7 +5798,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -5808,11 +5808,11 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>14</v>
+        <v>86</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,7 +5823,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -5833,11 +5833,11 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>86</v>
+        <v>14</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5898,7 +5898,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5908,11 +5908,11 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,7 +5923,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -5933,11 +5933,11 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -6023,7 +6023,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>17:58:44</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -6033,11 +6033,11 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,7 +6048,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -6058,11 +6058,11 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6258,7 +6258,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D237" t="n">
@@ -6283,7 +6283,7 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D238" t="n">
@@ -6398,7 +6398,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>18:38:18</t>
+          <t>18:53:19</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -6412,7 +6412,7 @@
         </is>
       </c>
       <c r="D243" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -6448,7 +6448,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>18:38:18</t>
+          <t>18:53:19</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -6462,7 +6462,7 @@
         </is>
       </c>
       <c r="D245" t="n">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6473,21 +6473,21 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>18:38:18</t>
+          <t>18:53:19</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>19:11</t>
+          <t>19:04</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6498,12 +6498,12 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>17:58:44</t>
+          <t>18:53:19</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>19:15</t>
+          <t>19:11</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -6512,7 +6512,7 @@
         </is>
       </c>
       <c r="D247" t="n">
-        <v>77</v>
+        <v>18</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6528,16 +6528,16 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:15</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6548,7 +6548,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>18:38:18</t>
+          <t>18:53:19</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -6562,7 +6562,7 @@
         </is>
       </c>
       <c r="D249" t="n">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -6573,7 +6573,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>18:18:08</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -6583,11 +6583,11 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6598,21 +6598,21 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>18:38:18</t>
+          <t>18:18:08</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>39</v>
+        <v>58</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -6623,21 +6623,21 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>18:38:18</t>
+          <t>18:53:19</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>46</v>
+        <v>24</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,21 +6648,21 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>18:53:19</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>19:26</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>102</v>
+        <v>31</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6673,12 +6673,12 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>18:18:08</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>19:27</t>
+          <t>19:26</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
@@ -6687,7 +6687,7 @@
         </is>
       </c>
       <c r="D254" t="n">
-        <v>69</v>
+        <v>102</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -6698,12 +6698,12 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>18:38:18</t>
+          <t>18:18:08</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>19:27</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
@@ -6712,7 +6712,7 @@
         </is>
       </c>
       <c r="D255" t="n">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6728,16 +6728,16 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>19:49</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6748,21 +6748,21 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>18:38:18</t>
+          <t>18:53:19</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>19:50</t>
+          <t>19:31</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D257" t="n">
-        <v>72</v>
+        <v>38</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -6773,21 +6773,21 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>18:38:18</t>
+          <t>18:53:19</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:49</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>83</v>
+        <v>56</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -6798,21 +6798,21 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>18:38:18</t>
+          <t>18:53:19</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>20:07</t>
+          <t>19:50</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D259" t="n">
-        <v>89</v>
+        <v>57</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -6823,21 +6823,21 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>18:38:18</t>
+          <t>18:53:19</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>19:56</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D260" t="n">
-        <v>97</v>
+        <v>63</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -6848,23 +6848,148 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
+          <t>18:53:19</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>20:01</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D261" t="n">
+        <v>68</v>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
           <t>18:38:18</t>
         </is>
       </c>
-      <c r="B261" t="inlineStr">
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>20:07</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D262" t="n">
+        <v>89</v>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>18:53:19</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
         <is>
           <t>20:15</t>
         </is>
       </c>
-      <c r="C261" t="inlineStr">
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D263" t="n">
+        <v>82</v>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>18:53:19</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D261" t="n">
-        <v>97</v>
-      </c>
-      <c r="E261" t="inlineStr">
+      <c r="D264" t="n">
+        <v>82</v>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>18:53:19</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D265" t="n">
+        <v>106</v>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>18:53:19</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D266" t="n">
+        <v>108</v>
+      </c>
+      <c r="E266" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6881,7 +7006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6894,14 +7019,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:38:18</t>
+          <t>Última actualización: 18:53:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 39</t>
+          <t>Total filas: 42</t>
         </is>
       </c>
     </row>
@@ -7070,7 +7195,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -7095,7 +7220,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -7785,7 +7910,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>18:38:18</t>
+          <t>18:53:19</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -7799,7 +7924,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -7885,23 +8010,98 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>18:38:18</t>
+          <t>18:53:19</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
+          <t>19:31</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>38</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>18:53:19</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
           <t>20:15</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D44" t="n">
-        <v>97</v>
-      </c>
-      <c r="E44" t="inlineStr">
+      <c r="D45" t="n">
+        <v>82</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>18:53:19</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>106</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>18:53:19</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>108</v>
+      </c>
+      <c r="E47" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7931,7 +8131,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:38:18</t>
+          <t>Última actualización: 18:53:19</t>
         </is>
       </c>
     </row>
@@ -8922,7 +9122,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>18:38:18</t>
+          <t>18:53:19</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -8936,7 +9136,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -8972,7 +9172,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>18:38:18</t>
+          <t>18:53:19</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -8986,7 +9186,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4677
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E266"/>
+  <dimension ref="A1:E276"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:53:19</t>
+          <t>Última actualización: 19:09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 261</t>
+          <t>Total filas: 271</t>
         </is>
       </c>
     </row>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>33</v>
+        <v>74</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>21</v>
+        <v>81</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>53</v>
+        <v>113</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3783,11 +3783,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>113</v>
+        <v>53</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3958,11 +3958,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>100</v>
+        <v>63</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>13</v>
+        <v>64</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -4008,7 +4008,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>64</v>
+        <v>13</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>83</v>
+        <v>34</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>103</v>
+        <v>61</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5773,7 +5773,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>15:49:32</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -5783,11 +5783,11 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>61</v>
+        <v>103</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -6023,7 +6023,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -6033,11 +6033,11 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,7 +6048,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>17:58:44</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -6058,11 +6058,11 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6258,7 +6258,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D237" t="n">
@@ -6283,7 +6283,7 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D238" t="n">
@@ -6523,12 +6523,12 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>17:58:44</t>
+          <t>19:09:00</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>19:15</t>
+          <t>19:12</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
@@ -6537,7 +6537,7 @@
         </is>
       </c>
       <c r="D248" t="n">
-        <v>77</v>
+        <v>3</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6548,21 +6548,21 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>18:53:19</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:15</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>23</v>
+        <v>77</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -6573,7 +6573,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>17:58:44</t>
+          <t>19:09:00</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -6583,11 +6583,11 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>78</v>
+        <v>7</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6598,7 +6598,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>18:18:08</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -6608,11 +6608,11 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -6623,21 +6623,21 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>18:53:19</t>
+          <t>18:18:08</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>24</v>
+        <v>58</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,21 +6648,21 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>18:53:19</t>
+          <t>19:09:00</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6673,21 +6673,21 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>19:09:00</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>19:26</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>102</v>
+        <v>15</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -6698,21 +6698,21 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>18:18:08</t>
+          <t>19:09:00</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>19:27</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6723,12 +6723,12 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>18:38:18</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>19:26</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -6737,7 +6737,7 @@
         </is>
       </c>
       <c r="D256" t="n">
-        <v>52</v>
+        <v>102</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6748,12 +6748,12 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>18:53:19</t>
+          <t>18:18:08</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>19:31</t>
+          <t>19:27</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
@@ -6762,7 +6762,7 @@
         </is>
       </c>
       <c r="D257" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -6773,21 +6773,21 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>18:53:19</t>
+          <t>19:09:00</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>19:49</t>
+          <t>19:29</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>56</v>
+        <v>20</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -6798,21 +6798,21 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>18:53:19</t>
+          <t>18:38:18</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>19:50</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D259" t="n">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -6828,16 +6828,16 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>19:56</t>
+          <t>19:31</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D260" t="n">
-        <v>63</v>
+        <v>38</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -6848,21 +6848,21 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>18:53:19</t>
+          <t>19:09:00</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:49</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D261" t="n">
-        <v>68</v>
+        <v>40</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -6873,21 +6873,21 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>18:38:18</t>
+          <t>19:09:00</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>20:07</t>
+          <t>19:50</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>89</v>
+        <v>41</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6898,21 +6898,21 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>18:53:19</t>
+          <t>19:09:00</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>19:56</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D263" t="n">
-        <v>82</v>
+        <v>47</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
@@ -6928,16 +6928,16 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6948,21 +6948,21 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>18:53:19</t>
+          <t>19:09:00</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:02</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>106</v>
+        <v>53</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -6973,23 +6973,273 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
+          <t>18:38:18</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>20:07</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D266" t="n">
+        <v>89</v>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
           <t>18:53:19</t>
         </is>
       </c>
-      <c r="B266" t="inlineStr">
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D267" t="n">
+        <v>82</v>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>19:09:00</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D268" t="n">
+        <v>66</v>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>19:09:00</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>20:16</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D269" t="n">
+        <v>67</v>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>18:53:19</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D270" t="n">
+        <v>106</v>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>19:09:00</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D271" t="n">
+        <v>91</v>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>18:53:19</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
         <is>
           <t>20:41</t>
         </is>
       </c>
-      <c r="C266" t="inlineStr">
+      <c r="C272" t="inlineStr">
         <is>
           <t>215_ALUAR</t>
         </is>
       </c>
-      <c r="D266" t="n">
+      <c r="D272" t="n">
         <v>108</v>
       </c>
-      <c r="E266" t="inlineStr">
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>19:09:00</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D273" t="n">
+        <v>93</v>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>19:09:00</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D274" t="n">
+        <v>108</v>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>19:09:00</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D275" t="n">
+        <v>117</v>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>19:09:00</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>21:07</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D276" t="n">
+        <v>118</v>
+      </c>
+      <c r="E276" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7006,7 +7256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7019,14 +7269,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:53:19</t>
+          <t>Última actualización: 19:09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 42</t>
+          <t>Total filas: 46</t>
         </is>
       </c>
     </row>
@@ -7195,7 +7445,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -7220,7 +7470,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -7985,12 +8235,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>18:38:18</t>
+          <t>19:09:00</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>19:29</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -7999,7 +8249,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>52</v>
+        <v>20</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -8010,12 +8260,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>18:53:19</t>
+          <t>18:38:18</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>19:31</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -8024,7 +8274,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -8040,7 +8290,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>19:31</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -8049,7 +8299,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>82</v>
+        <v>38</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -8060,21 +8310,21 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>18:53:19</t>
+          <t>19:09:00</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>106</v>
+        <v>66</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -8090,18 +8340,118 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>106</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>19:09:00</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>91</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>18:53:19</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
           <t>20:41</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>215_ALUAR</t>
         </is>
       </c>
-      <c r="D47" t="n">
+      <c r="D49" t="n">
         <v>108</v>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>19:09:00</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>93</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>19:09:00</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>21:07</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>118</v>
+      </c>
+      <c r="E51" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8118,7 +8468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8131,14 +8481,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:53:19</t>
+          <t>Última actualización: 19:09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 41</t>
+          <t>Total filas: 42</t>
         </is>
       </c>
     </row>
@@ -9122,7 +9472,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>18:53:19</t>
+          <t>19:09:00</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -9136,7 +9486,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -9172,7 +9522,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>18:53:19</t>
+          <t>19:09:00</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -9186,9 +9536,34 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="E46" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>19:09:00</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>107</v>
+      </c>
+      <c r="E47" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4678
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E276"/>
+  <dimension ref="A1:E279"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:09:00</t>
+          <t>Última actualización: 19:34:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 271</t>
+          <t>Total filas: 274</t>
         </is>
       </c>
     </row>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1533,11 +1533,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>21</v>
+        <v>81</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>100</v>
+        <v>63</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3958,7 +3958,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>64</v>
+        <v>13</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>13</v>
+        <v>64</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -5798,7 +5798,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -5808,11 +5808,11 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>86</v>
+        <v>14</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,7 +5823,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -5833,11 +5833,11 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>14</v>
+        <v>86</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -6258,7 +6258,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D237" t="n">
@@ -6283,7 +6283,7 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D238" t="n">
@@ -6573,7 +6573,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>19:09:00</t>
+          <t>18:18:08</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -6583,11 +6583,11 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>7</v>
+        <v>58</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6623,7 +6623,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>18:18:08</t>
+          <t>19:09:00</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -6633,11 +6633,11 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>58</v>
+        <v>7</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6848,7 +6848,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>19:09:00</t>
+          <t>19:34:24</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
@@ -6862,7 +6862,7 @@
         </is>
       </c>
       <c r="D261" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -6873,7 +6873,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>19:09:00</t>
+          <t>19:34:24</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -6887,7 +6887,7 @@
         </is>
       </c>
       <c r="D262" t="n">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6898,7 +6898,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>19:09:00</t>
+          <t>19:34:24</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
@@ -6912,7 +6912,7 @@
         </is>
       </c>
       <c r="D263" t="n">
-        <v>47</v>
+        <v>22</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
@@ -6923,7 +6923,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>18:53:19</t>
+          <t>19:34:24</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -6937,7 +6937,7 @@
         </is>
       </c>
       <c r="D264" t="n">
-        <v>68</v>
+        <v>27</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6998,7 +6998,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>18:53:19</t>
+          <t>19:34:24</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -7008,11 +7008,11 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>82</v>
+        <v>41</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7023,7 +7023,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>19:09:00</t>
+          <t>19:34:24</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -7033,11 +7033,11 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>66</v>
+        <v>41</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7073,21 +7073,21 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>18:53:19</t>
+          <t>19:34:24</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:36</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D270" t="n">
-        <v>106</v>
+        <v>62</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7098,12 +7098,12 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>19:09:00</t>
+          <t>19:34:24</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>20:40</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
@@ -7112,7 +7112,7 @@
         </is>
       </c>
       <c r="D271" t="n">
-        <v>91</v>
+        <v>65</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,21 +7123,21 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>18:53:19</t>
+          <t>19:09:00</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:40</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>108</v>
+        <v>91</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7148,12 +7148,12 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>19:09:00</t>
+          <t>19:34:24</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>20:42</t>
+          <t>20:41</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
@@ -7162,7 +7162,7 @@
         </is>
       </c>
       <c r="D273" t="n">
-        <v>93</v>
+        <v>67</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7178,16 +7178,16 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:42</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>108</v>
+        <v>93</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7198,21 +7198,21 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>19:09:00</t>
+          <t>19:34:24</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>117</v>
+        <v>83</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7223,23 +7223,98 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
+          <t>19:34:24</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>20:59</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D276" t="n">
+        <v>85</v>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>19:34:24</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D277" t="n">
+        <v>92</v>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>19:34:24</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D278" t="n">
+        <v>92</v>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
           <t>19:09:00</t>
         </is>
       </c>
-      <c r="B276" t="inlineStr">
+      <c r="B279" t="inlineStr">
         <is>
           <t>21:07</t>
         </is>
       </c>
-      <c r="C276" t="inlineStr">
+      <c r="C279" t="inlineStr">
         <is>
           <t>215_ALUAR</t>
         </is>
       </c>
-      <c r="D276" t="n">
+      <c r="D279" t="n">
         <v>118</v>
       </c>
-      <c r="E276" t="inlineStr">
+      <c r="E279" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7256,7 +7331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7269,14 +7344,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:09:00</t>
+          <t>Última actualización: 19:34:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 46</t>
+          <t>Total filas: 47</t>
         </is>
       </c>
     </row>
@@ -7445,7 +7520,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -7470,7 +7545,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -8310,7 +8385,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>19:09:00</t>
+          <t>19:34:24</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -8324,7 +8399,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>66</v>
+        <v>41</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -8335,7 +8410,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>18:53:19</t>
+          <t>19:34:24</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -8349,7 +8424,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>106</v>
+        <v>65</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -8385,7 +8460,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>18:53:19</t>
+          <t>19:34:24</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -8399,7 +8474,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>108</v>
+        <v>67</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -8435,23 +8510,48 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t>19:34:24</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>92</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
           <t>19:09:00</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B52" t="inlineStr">
         <is>
           <t>21:07</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C52" t="inlineStr">
         <is>
           <t>215_ALUAR</t>
         </is>
       </c>
-      <c r="D51" t="n">
+      <c r="D52" t="n">
         <v>118</v>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="E52" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8468,7 +8568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8481,14 +8581,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:09:00</t>
+          <t>Última actualización: 19:34:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 42</t>
+          <t>Total filas: 43</t>
         </is>
       </c>
     </row>
@@ -9522,7 +9622,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>19:09:00</t>
+          <t>19:34:24</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -9536,7 +9636,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -9564,6 +9664,31 @@
         <v>107</v>
       </c>
       <c r="E47" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>19:34:24</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>21:32</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>118</v>
+      </c>
+      <c r="E48" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4679
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E279"/>
+  <dimension ref="A1:E285"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:34:24</t>
+          <t>Última actualización: 19:52:22</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 274</t>
+          <t>Total filas: 280</t>
         </is>
       </c>
     </row>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1533,11 +1533,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>33</v>
+        <v>74</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>59</v>
+        <v>12</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>10:46:10</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2633,11 +2633,11 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>12</v>
+        <v>59</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>91</v>
+        <v>32</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>32</v>
+        <v>91</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>113</v>
+        <v>53</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3783,11 +3783,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>53</v>
+        <v>113</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>100</v>
+        <v>63</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3933,7 +3933,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3958,11 +3958,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>13</v>
+        <v>64</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>64</v>
+        <v>13</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>15:49:32</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>61</v>
+        <v>103</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5773,7 +5773,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -5783,11 +5783,11 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>103</v>
+        <v>61</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,7 +5798,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -5808,11 +5808,11 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>14</v>
+        <v>86</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,7 +5823,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -5833,11 +5833,11 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>86</v>
+        <v>14</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -6898,21 +6898,21 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>19:34:24</t>
+          <t>19:52:22</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>19:56</t>
+          <t>19:53</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D263" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
@@ -6923,21 +6923,21 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>19:34:24</t>
+          <t>19:52:22</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:53</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6948,21 +6948,21 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>19:09:00</t>
+          <t>19:52:22</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>19:56</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>53</v>
+        <v>4</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -6973,21 +6973,21 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>18:38:18</t>
+          <t>19:52:22</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>20:07</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>89</v>
+        <v>9</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -6998,21 +6998,21 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>19:34:24</t>
+          <t>19:09:00</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:02</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7023,21 +7023,21 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>19:34:24</t>
+          <t>18:38:18</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:07</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>41</v>
+        <v>89</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7048,12 +7048,12 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>19:09:00</t>
+          <t>19:34:24</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>20:16</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -7062,7 +7062,7 @@
         </is>
       </c>
       <c r="D269" t="n">
-        <v>67</v>
+        <v>41</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7073,21 +7073,21 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>19:34:24</t>
+          <t>19:52:22</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>20:36</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D270" t="n">
-        <v>62</v>
+        <v>23</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7098,21 +7098,21 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>19:34:24</t>
+          <t>19:09:00</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:16</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,21 +7123,21 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>19:09:00</t>
+          <t>19:52:22</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>20:40</t>
+          <t>20:36</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>91</v>
+        <v>44</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7148,21 +7148,21 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>19:34:24</t>
+          <t>19:52:22</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>67</v>
+        <v>47</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7178,16 +7178,16 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>20:42</t>
+          <t>20:40</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7198,21 +7198,21 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>19:34:24</t>
+          <t>19:52:22</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:41</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>83</v>
+        <v>49</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7223,21 +7223,21 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>19:34:24</t>
+          <t>19:09:00</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>20:59</t>
+          <t>20:42</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D276" t="n">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -7248,21 +7248,21 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>19:34:24</t>
+          <t>19:52:22</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>20:47</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D277" t="n">
-        <v>92</v>
+        <v>55</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -7273,21 +7273,21 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>19:34:24</t>
+          <t>19:52:22</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>92</v>
+        <v>65</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7298,23 +7298,173 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
+          <t>19:34:24</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>20:59</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D279" t="n">
+        <v>85</v>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>19:52:22</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>21:04</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D280" t="n">
+        <v>72</v>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>19:52:22</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D281" t="n">
+        <v>74</v>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>19:52:22</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D282" t="n">
+        <v>74</v>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
           <t>19:09:00</t>
         </is>
       </c>
-      <c r="B279" t="inlineStr">
+      <c r="B283" t="inlineStr">
         <is>
           <t>21:07</t>
         </is>
       </c>
-      <c r="C279" t="inlineStr">
+      <c r="C283" t="inlineStr">
         <is>
           <t>215_ALUAR</t>
         </is>
       </c>
-      <c r="D279" t="n">
+      <c r="D283" t="n">
         <v>118</v>
       </c>
-      <c r="E279" t="inlineStr">
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>19:52:22</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D284" t="n">
+        <v>102</v>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>19:52:22</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>21:37</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D285" t="n">
+        <v>105</v>
+      </c>
+      <c r="E285" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7344,7 +7494,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:34:24</t>
+          <t>Última actualización: 19:52:22</t>
         </is>
       </c>
     </row>
@@ -7520,7 +7670,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -7545,7 +7695,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -8385,7 +8535,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>19:34:24</t>
+          <t>19:52:22</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -8399,7 +8549,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -8410,7 +8560,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>19:34:24</t>
+          <t>19:52:22</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -8424,7 +8574,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>65</v>
+        <v>47</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -8460,7 +8610,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>19:34:24</t>
+          <t>19:52:22</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -8474,7 +8624,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -8510,7 +8660,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>19:34:24</t>
+          <t>19:52:22</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -8524,7 +8674,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>92</v>
+        <v>74</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -8568,7 +8718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8581,14 +8731,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:34:24</t>
+          <t>Última actualización: 19:52:22</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 43</t>
+          <t>Total filas: 44</t>
         </is>
       </c>
     </row>
@@ -9647,12 +9797,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>19:09:00</t>
+          <t>19:52:22</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -9661,7 +9811,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>107</v>
+        <v>47</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -9672,23 +9822,48 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>19:34:24</t>
+          <t>19:09:00</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>107</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>19:52:22</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
           <t>21:32</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D48" t="n">
-        <v>118</v>
-      </c>
-      <c r="E48" t="inlineStr">
+      <c r="D49" t="n">
+        <v>100</v>
+      </c>
+      <c r="E49" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4680
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E285"/>
+  <dimension ref="A1:E294"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:52:22</t>
+          <t>Última actualización: 20:09:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 280</t>
+          <t>Total filas: 289</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>45</v>
+        <v>105</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>105</v>
+        <v>45</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1533,11 +1533,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:58:16</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:58:16</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>33</v>
+        <v>74</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>53</v>
+        <v>113</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3783,11 +3783,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>113</v>
+        <v>53</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3958,11 +3958,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>100</v>
+        <v>63</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>64</v>
+        <v>13</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,7 +3998,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4008,11 +4008,11 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>13</v>
+        <v>64</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4033,7 +4033,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>83</v>
+        <v>34</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>15:49:32</t>
+          <t>16:31:13</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>103</v>
+        <v>61</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5773,7 +5773,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>16:31:13</t>
+          <t>15:49:32</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -5783,11 +5783,11 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>61</v>
+        <v>103</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,7 +5798,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -5808,11 +5808,11 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>86</v>
+        <v>14</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,7 +5823,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -5833,11 +5833,11 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>14</v>
+        <v>86</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -6023,7 +6023,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>17:58:44</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -6033,11 +6033,11 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,7 +6048,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -6058,11 +6058,11 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6258,7 +6258,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D237" t="n">
@@ -6283,7 +6283,7 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D238" t="n">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D254" t="n">
@@ -6708,7 +6708,7 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D255" t="n">
@@ -7048,21 +7048,21 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>19:34:24</t>
+          <t>20:09:31</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:12</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>41</v>
+        <v>3</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7073,7 +7073,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>19:52:22</t>
+          <t>20:09:31</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -7087,7 +7087,7 @@
         </is>
       </c>
       <c r="D270" t="n">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7098,12 +7098,12 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>19:09:00</t>
+          <t>20:09:31</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>20:16</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
@@ -7112,7 +7112,7 @@
         </is>
       </c>
       <c r="D271" t="n">
-        <v>67</v>
+        <v>6</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,21 +7123,21 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>19:52:22</t>
+          <t>19:09:00</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>20:36</t>
+          <t>20:16</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7148,21 +7148,21 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>19:52:22</t>
+          <t>20:09:31</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:36</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>47</v>
+        <v>27</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7173,12 +7173,12 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>19:09:00</t>
+          <t>20:09:31</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>20:40</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
@@ -7187,7 +7187,7 @@
         </is>
       </c>
       <c r="D274" t="n">
-        <v>91</v>
+        <v>30</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7198,21 +7198,21 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>19:52:22</t>
+          <t>19:09:00</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:40</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>49</v>
+        <v>91</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7223,12 +7223,12 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>19:09:00</t>
+          <t>20:09:31</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>20:42</t>
+          <t>20:41</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -7237,7 +7237,7 @@
         </is>
       </c>
       <c r="D276" t="n">
-        <v>93</v>
+        <v>32</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -7248,21 +7248,21 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>19:52:22</t>
+          <t>19:09:00</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>20:47</t>
+          <t>20:42</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D277" t="n">
-        <v>55</v>
+        <v>93</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -7278,16 +7278,16 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:47</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7298,21 +7298,21 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>19:34:24</t>
+          <t>20:09:31</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>20:59</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>85</v>
+        <v>47</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7328,16 +7328,16 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>21:04</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7348,21 +7348,21 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>19:52:22</t>
+          <t>19:34:24</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>20:59</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>74</v>
+        <v>85</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7373,21 +7373,21 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>19:52:22</t>
+          <t>20:09:31</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>21:02</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>74</v>
+        <v>53</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7398,21 +7398,21 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>19:09:00</t>
+          <t>19:52:22</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>21:07</t>
+          <t>21:04</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>118</v>
+        <v>72</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -7423,21 +7423,21 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>19:52:22</t>
+          <t>20:09:31</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:05</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D284" t="n">
-        <v>102</v>
+        <v>56</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -7453,18 +7453,243 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D285" t="n">
+        <v>74</v>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>20:09:31</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D286" t="n">
+        <v>57</v>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>19:09:00</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>21:07</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D287" t="n">
+        <v>118</v>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>20:09:31</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>21:16</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D288" t="n">
+        <v>67</v>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>20:09:31</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D289" t="n">
+        <v>85</v>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>20:09:31</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D290" t="n">
+        <v>87</v>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>20:09:31</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
           <t>21:37</t>
         </is>
       </c>
-      <c r="C285" t="inlineStr">
+      <c r="C291" t="inlineStr">
         <is>
           <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
-      <c r="D285" t="n">
-        <v>105</v>
-      </c>
-      <c r="E285" t="inlineStr">
+      <c r="D291" t="n">
+        <v>88</v>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>20:09:31</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>21:39</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D292" t="n">
+        <v>90</v>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>20:09:31</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>21:59</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D293" t="n">
+        <v>110</v>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>20:09:31</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>22:07</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D294" t="n">
+        <v>118</v>
+      </c>
+      <c r="E294" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7494,7 +7719,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:52:22</t>
+          <t>Última actualización: 20:09:31</t>
         </is>
       </c>
     </row>
@@ -7670,7 +7895,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -7695,7 +7920,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -8535,7 +8760,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>19:52:22</t>
+          <t>20:09:31</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -8549,7 +8774,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -8560,7 +8785,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>19:52:22</t>
+          <t>20:09:31</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -8574,7 +8799,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -8610,7 +8835,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>19:52:22</t>
+          <t>20:09:31</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -8624,7 +8849,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -8660,7 +8885,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>19:52:22</t>
+          <t>20:09:31</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -8674,7 +8899,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -8731,7 +8956,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:52:22</t>
+          <t>Última actualización: 20:09:31</t>
         </is>
       </c>
     </row>
@@ -9797,7 +10022,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>19:52:22</t>
+          <t>20:09:31</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -9811,7 +10036,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -9847,7 +10072,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>19:52:22</t>
+          <t>20:09:31</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -9861,7 +10086,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4681
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E294"/>
+  <dimension ref="A1:E298"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:09:31</t>
+          <t>Última actualización: 20:32:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 289</t>
+          <t>Total filas: 293</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07:00:10</t>
+          <t>08:00:25</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>105</v>
+        <v>45</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:00:25</t>
+          <t>07:00:10</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>45</v>
+        <v>105</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>33</v>
+        <v>74</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>10:46:10</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>12</v>
+        <v>59</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2633,11 +2633,11 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>59</v>
+        <v>12</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>32</v>
+        <v>91</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>91</v>
+        <v>32</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>21</v>
+        <v>81</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>113</v>
+        <v>53</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3783,11 +3783,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>53</v>
+        <v>113</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>100</v>
+        <v>63</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3958,7 +3958,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>13</v>
+        <v>64</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,7 +3998,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4008,11 +4008,11 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>64</v>
+        <v>13</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -4508,7 +4508,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -5798,7 +5798,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -5808,11 +5808,11 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>14</v>
+        <v>86</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,7 +5823,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -5833,11 +5833,11 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>86</v>
+        <v>14</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5898,7 +5898,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5908,11 +5908,11 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,7 +5923,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -5933,11 +5933,11 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -6598,7 +6598,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>17:58:44</t>
+          <t>19:09:00</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -6608,11 +6608,11 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>78</v>
+        <v>7</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -6623,7 +6623,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>19:09:00</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -6633,11 +6633,11 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>7</v>
+        <v>78</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6683,7 +6683,7 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D254" t="n">
@@ -6708,7 +6708,7 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D255" t="n">
@@ -7148,7 +7148,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>20:09:31</t>
+          <t>20:32:38</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -7162,7 +7162,7 @@
         </is>
       </c>
       <c r="D273" t="n">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7173,7 +7173,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>20:09:31</t>
+          <t>20:32:38</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
@@ -7187,7 +7187,7 @@
         </is>
       </c>
       <c r="D274" t="n">
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7223,7 +7223,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>20:09:31</t>
+          <t>20:32:38</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
@@ -7237,7 +7237,7 @@
         </is>
       </c>
       <c r="D276" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -7298,21 +7298,21 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>20:09:31</t>
+          <t>20:32:38</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>47</v>
+        <v>19</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7323,12 +7323,12 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>19:52:22</t>
+          <t>20:32:38</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -7337,7 +7337,7 @@
         </is>
       </c>
       <c r="D280" t="n">
-        <v>65</v>
+        <v>24</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7348,21 +7348,21 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>19:34:24</t>
+          <t>19:52:22</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>20:59</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7373,12 +7373,12 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>20:09:31</t>
+          <t>19:34:24</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>21:02</t>
+          <t>20:59</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -7387,7 +7387,7 @@
         </is>
       </c>
       <c r="D282" t="n">
-        <v>53</v>
+        <v>85</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7398,12 +7398,12 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>19:52:22</t>
+          <t>20:09:31</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>21:04</t>
+          <t>21:02</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -7412,7 +7412,7 @@
         </is>
       </c>
       <c r="D283" t="n">
-        <v>72</v>
+        <v>53</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -7423,21 +7423,21 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>20:09:31</t>
+          <t>19:52:22</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>21:05</t>
+          <t>21:04</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D284" t="n">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -7448,12 +7448,12 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>19:52:22</t>
+          <t>20:32:38</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>21:05</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -7462,7 +7462,7 @@
         </is>
       </c>
       <c r="D285" t="n">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -7473,7 +7473,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>20:09:31</t>
+          <t>20:32:38</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
@@ -7487,7 +7487,7 @@
         </is>
       </c>
       <c r="D286" t="n">
-        <v>57</v>
+        <v>34</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -7498,21 +7498,21 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>19:09:00</t>
+          <t>19:52:22</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>21:07</t>
+          <t>21:06</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>118</v>
+        <v>74</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -7523,21 +7523,21 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>20:09:31</t>
+          <t>19:09:00</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>21:16</t>
+          <t>21:07</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>67</v>
+        <v>118</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7553,16 +7553,16 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:16</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7573,21 +7573,21 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>20:09:31</t>
+          <t>20:32:38</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>21:36</t>
+          <t>21:34</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>87</v>
+        <v>62</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7598,21 +7598,21 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>20:09:31</t>
+          <t>20:32:38</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>21:37</t>
+          <t>21:35</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -7628,16 +7628,16 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>21:39</t>
+          <t>21:36</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7648,21 +7648,21 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>20:09:31</t>
+          <t>20:32:38</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>21:59</t>
+          <t>21:37</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>110</v>
+        <v>65</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7678,18 +7678,118 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
+          <t>21:39</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D294" t="n">
+        <v>90</v>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>20:32:38</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>21:45</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D295" t="n">
+        <v>73</v>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>20:32:38</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>21:58</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D296" t="n">
+        <v>86</v>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>20:09:31</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>21:59</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D297" t="n">
+        <v>110</v>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>20:32:38</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
           <t>22:07</t>
         </is>
       </c>
-      <c r="C294" t="inlineStr">
+      <c r="C298" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D294" t="n">
-        <v>118</v>
-      </c>
-      <c r="E294" t="inlineStr">
+      <c r="D298" t="n">
+        <v>95</v>
+      </c>
+      <c r="E298" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7719,7 +7819,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:09:31</t>
+          <t>Última actualización: 20:32:38</t>
         </is>
       </c>
     </row>
@@ -7895,7 +7995,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -7920,7 +8020,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -8785,7 +8885,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>20:09:31</t>
+          <t>20:32:38</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -8799,7 +8899,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -8835,7 +8935,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>20:09:31</t>
+          <t>20:32:38</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -8849,7 +8949,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -8885,7 +8985,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>20:09:31</t>
+          <t>20:32:38</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -8899,7 +8999,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>57</v>
+        <v>34</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -8943,7 +9043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8956,14 +9056,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:09:31</t>
+          <t>Última actualización: 20:32:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 44</t>
+          <t>Total filas: 47</t>
         </is>
       </c>
     </row>
@@ -10022,12 +10122,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>20:09:31</t>
+          <t>20:32:38</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:38</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -10036,7 +10136,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -10047,12 +10147,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>19:09:00</t>
+          <t>20:09:31</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -10061,7 +10161,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>107</v>
+        <v>30</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -10072,25 +10172,100 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
+          <t>19:09:00</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>107</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>20:32:38</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>21:31</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>59</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t>20:09:31</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>21:32</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D49" t="n">
+      <c r="D51" t="n">
         <v>83</v>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E51" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>20:32:38</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>22:08</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>96</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4682
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E298"/>
+  <dimension ref="A1:E302"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:32:38</t>
+          <t>Última actualización: 20:51:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 293</t>
+          <t>Total filas: 297</t>
         </is>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>09:31:22</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>33</v>
+        <v>74</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:31:22</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>21</v>
+        <v>81</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>53</v>
+        <v>113</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3783,11 +3783,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>113</v>
+        <v>53</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3933,7 +3933,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -3958,7 +3958,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>64</v>
+        <v>13</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,7 +3998,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4008,11 +4008,11 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>13</v>
+        <v>64</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -4508,7 +4508,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>83</v>
+        <v>34</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -6573,7 +6573,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>18:18:08</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -6583,11 +6583,11 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6598,7 +6598,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>19:09:00</t>
+          <t>18:18:08</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -6608,11 +6608,11 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>7</v>
+        <v>58</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -6623,7 +6623,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>17:58:44</t>
+          <t>19:09:00</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -6633,11 +6633,11 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>78</v>
+        <v>7</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6908,7 +6908,7 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D263" t="n">
@@ -6933,7 +6933,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D264" t="n">
@@ -7083,7 +7083,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D270" t="n">
@@ -7108,7 +7108,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D271" t="n">
@@ -7298,7 +7298,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>20:32:38</t>
+          <t>20:51:14</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
@@ -7312,7 +7312,7 @@
         </is>
       </c>
       <c r="D279" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7348,7 +7348,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>19:52:22</t>
+          <t>20:51:14</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
@@ -7362,7 +7362,7 @@
         </is>
       </c>
       <c r="D281" t="n">
-        <v>65</v>
+        <v>6</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7473,7 +7473,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>20:32:38</t>
+          <t>20:51:14</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
@@ -7483,11 +7483,11 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -7498,7 +7498,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>19:52:22</t>
+          <t>20:51:14</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
@@ -7508,11 +7508,11 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>74</v>
+        <v>15</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -7573,7 +7573,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>20:32:38</t>
+          <t>20:51:14</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
@@ -7587,7 +7587,7 @@
         </is>
       </c>
       <c r="D290" t="n">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7623,7 +7623,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>20:09:31</t>
+          <t>20:51:14</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
@@ -7637,7 +7637,7 @@
         </is>
       </c>
       <c r="D292" t="n">
-        <v>87</v>
+        <v>45</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>20:32:38</t>
+          <t>20:51:14</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7662,7 +7662,7 @@
         </is>
       </c>
       <c r="D293" t="n">
-        <v>65</v>
+        <v>46</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7698,12 +7698,12 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>20:32:38</t>
+          <t>20:51:14</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>21:40</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -7712,7 +7712,7 @@
         </is>
       </c>
       <c r="D295" t="n">
-        <v>73</v>
+        <v>49</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7728,16 +7728,16 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>21:58</t>
+          <t>21:45</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>86</v>
+        <v>73</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -7748,12 +7748,12 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>20:09:31</t>
+          <t>20:32:38</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>21:59</t>
+          <t>21:58</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -7762,7 +7762,7 @@
         </is>
       </c>
       <c r="D297" t="n">
-        <v>110</v>
+        <v>86</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
@@ -7773,23 +7773,123 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>20:32:38</t>
+          <t>20:51:14</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
+          <t>21:59</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D298" t="n">
+        <v>68</v>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>20:51:14</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
           <t>22:07</t>
         </is>
       </c>
-      <c r="C298" t="inlineStr">
+      <c r="C299" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D298" t="n">
+      <c r="D299" t="n">
+        <v>76</v>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>20:51:14</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>22:26</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D300" t="n">
         <v>95</v>
       </c>
-      <c r="E298" t="inlineStr">
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>20:51:14</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>22:37</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D301" t="n">
+        <v>106</v>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>20:51:14</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>22:41</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D302" t="n">
+        <v>110</v>
+      </c>
+      <c r="E302" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7806,7 +7906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7819,14 +7919,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:32:38</t>
+          <t>Última actualización: 20:51:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 47</t>
+          <t>Total filas: 48</t>
         </is>
       </c>
     </row>
@@ -7995,7 +8095,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -8020,7 +8120,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -8985,7 +9085,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>20:32:38</t>
+          <t>20:51:14</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -8999,7 +9099,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -9027,6 +9127,31 @@
         <v>118</v>
       </c>
       <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>20:51:14</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>22:37</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>106</v>
+      </c>
+      <c r="E53" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9043,7 +9168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9056,14 +9181,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:32:38</t>
+          <t>Última actualización: 20:51:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 47</t>
+          <t>Total filas: 48</t>
         </is>
       </c>
     </row>
@@ -10222,7 +10347,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>20:09:31</t>
+          <t>20:51:14</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -10236,7 +10361,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>83</v>
+        <v>41</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -10264,6 +10389,31 @@
         <v>96</v>
       </c>
       <c r="E52" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>20:51:14</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>22:09</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>78</v>
+      </c>
+      <c r="E53" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4683
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E302"/>
+  <dimension ref="A1:E307"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:51:14</t>
+          <t>Última actualización: 21:33:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 297</t>
+          <t>Total filas: 302</t>
         </is>
       </c>
     </row>
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>59</v>
+        <v>12</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>10:46:10</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2633,11 +2633,11 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>12</v>
+        <v>59</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>113</v>
+        <v>53</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3783,11 +3783,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>53</v>
+        <v>113</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>100</v>
+        <v>63</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3958,7 +3958,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>13</v>
+        <v>64</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,7 +3998,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4008,11 +4008,11 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>64</v>
+        <v>13</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4033,7 +4033,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -4508,7 +4508,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>83</v>
+        <v>34</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -6023,7 +6023,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -6033,11 +6033,11 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,7 +6048,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>17:58:44</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -6058,11 +6058,11 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6573,7 +6573,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>17:58:44</t>
+          <t>19:09:00</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -6583,11 +6583,11 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>78</v>
+        <v>7</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6598,7 +6598,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>18:18:08</t>
+          <t>17:58:44</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -6608,11 +6608,11 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -6623,7 +6623,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>19:09:00</t>
+          <t>18:18:08</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -6633,11 +6633,11 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>7</v>
+        <v>58</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6908,7 +6908,7 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D263" t="n">
@@ -6933,7 +6933,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D264" t="n">
@@ -7573,21 +7573,21 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>20:51:14</t>
+          <t>21:33:35</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:33</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7598,21 +7598,21 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>20:32:38</t>
+          <t>20:51:14</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>21:35</t>
+          <t>21:34</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>63</v>
+        <v>43</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -7623,21 +7623,21 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>20:51:14</t>
+          <t>21:33:35</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>21:36</t>
+          <t>21:35</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>45</v>
+        <v>2</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7648,21 +7648,21 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>20:51:14</t>
+          <t>20:32:38</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>21:37</t>
+          <t>21:35</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,21 +7673,21 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>20:09:31</t>
+          <t>21:33:35</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>21:39</t>
+          <t>21:36</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>90</v>
+        <v>3</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7698,21 +7698,21 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>20:51:14</t>
+          <t>21:33:35</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>21:40</t>
+          <t>21:37</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>49</v>
+        <v>4</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,12 +7723,12 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>20:32:38</t>
+          <t>20:09:31</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>21:39</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -7737,7 +7737,7 @@
         </is>
       </c>
       <c r="D296" t="n">
-        <v>73</v>
+        <v>90</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -7748,21 +7748,21 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>20:32:38</t>
+          <t>21:33:35</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>21:58</t>
+          <t>21:40</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D297" t="n">
-        <v>86</v>
+        <v>7</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
@@ -7773,21 +7773,21 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>20:51:14</t>
+          <t>20:32:38</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>21:59</t>
+          <t>21:45</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D298" t="n">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="E298" t="inlineStr">
         <is>
@@ -7798,21 +7798,21 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>20:51:14</t>
+          <t>20:32:38</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>22:07</t>
+          <t>21:58</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -7823,21 +7823,21 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>20:51:14</t>
+          <t>21:33:35</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>22:26</t>
+          <t>21:59</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D300" t="n">
-        <v>95</v>
+        <v>26</v>
       </c>
       <c r="E300" t="inlineStr">
         <is>
@@ -7848,21 +7848,21 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>20:51:14</t>
+          <t>21:33:35</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>22:37</t>
+          <t>22:07</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D301" t="n">
-        <v>106</v>
+        <v>34</v>
       </c>
       <c r="E301" t="inlineStr">
         <is>
@@ -7873,23 +7873,148 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
+          <t>21:33:35</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>22:26</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D302" t="n">
+        <v>53</v>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
           <t>20:51:14</t>
         </is>
       </c>
-      <c r="B302" t="inlineStr">
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>22:37</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D303" t="n">
+        <v>106</v>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>21:33:35</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
         <is>
           <t>22:41</t>
         </is>
       </c>
-      <c r="C302" t="inlineStr">
+      <c r="C304" t="inlineStr">
         <is>
           <t>16_SANTA ANA</t>
         </is>
       </c>
-      <c r="D302" t="n">
-        <v>110</v>
-      </c>
-      <c r="E302" t="inlineStr">
+      <c r="D304" t="n">
+        <v>68</v>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>21:33:35</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>22:55</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D305" t="n">
+        <v>82</v>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>21:33:35</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>23:07</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D306" t="n">
+        <v>94</v>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>21:33:35</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>23:30</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D307" t="n">
+        <v>117</v>
+      </c>
+      <c r="E307" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7906,7 +8031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7919,14 +8044,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:51:14</t>
+          <t>Última actualización: 21:33:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 48</t>
+          <t>Total filas: 50</t>
         </is>
       </c>
     </row>
@@ -8095,7 +8220,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -8120,7 +8245,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -9135,23 +9260,73 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>21:33:35</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>21:33</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
           <t>20:51:14</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>22:37</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D53" t="n">
+      <c r="D54" t="n">
         <v>106</v>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>21:33:35</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>23:30</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>117</v>
+      </c>
+      <c r="E55" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9168,7 +9343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9181,14 +9356,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:51:14</t>
+          <t>Última actualización: 21:33:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 48</t>
+          <t>Total filas: 50</t>
         </is>
       </c>
     </row>
@@ -10372,50 +10547,100 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>20:32:38</t>
+          <t>21:33:35</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>22:08</t>
+          <t>21:34</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-40 Y 115</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>96</v>
+        <v>1</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>20:51:14</t>
+          <t>20:32:38</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
+          <t>22:08</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>96</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>21:33:35</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
           <t>22:09</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-40 Y 115</t>
         </is>
       </c>
-      <c r="D53" t="n">
-        <v>78</v>
-      </c>
-      <c r="E53" t="inlineStr">
+      <c r="D54" t="n">
+        <v>36</v>
+      </c>
+      <c r="E54" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>21:33:35</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>22:40</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>67</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4684
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-23.xlsx
+++ b/data/horarios-141-2026-08-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E307"/>
+  <dimension ref="A1:E312"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 21:33:35</t>
+          <t>Última actualización: 23:09:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 302</t>
+          <t>Total filas: 307</t>
         </is>
       </c>
     </row>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>10:16:16</t>
+          <t>08:29:38</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:29:38</t>
+          <t>10:16:16</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>11:33:07</t>
+          <t>10:46:10</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>12</v>
+        <v>59</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>10:46:10</t>
+          <t>11:33:07</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2633,11 +2633,11 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>59</v>
+        <v>12</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>11:53:55</t>
+          <t>12:52:01</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>91</v>
+        <v>32</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>12:52:01</t>
+          <t>11:53:55</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>32</v>
+        <v>91</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:10:06</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>21</v>
+        <v>81</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>12:10:06</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>12:33:46</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>12:33:46</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>100</v>
+        <v>63</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3958,7 +3958,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>13:10:57</t>
+          <t>14:01:31</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>64</v>
+        <v>13</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,7 +3998,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>14:01:31</t>
+          <t>13:10:57</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4008,11 +4008,11 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>13</v>
+        <v>64</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>15:17:10</t>
+          <t>14:28:51</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>14:28:51</t>
+          <t>15:17:10</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>83</v>
+        <v>34</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -5798,7 +5798,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>16:09:36</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -5808,11 +5808,11 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>86</v>
+        <v>14</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,7 +5823,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>16:09:36</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -5833,11 +5833,11 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>14</v>
+        <v>86</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5898,7 +5898,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>17:21:32</t>
+          <t>17:44:31</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5908,11 +5908,11 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,7 +5923,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>17:44:31</t>
+          <t>17:21:32</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -5933,11 +5933,11 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -6573,7 +6573,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>19:09:00</t>
+          <t>18:18:08</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -6583,11 +6583,11 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>7</v>
+        <v>58</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6623,7 +6623,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>18:18:08</t>
+          <t>19:09:00</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -6633,11 +6633,11 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>58</v>
+        <v>7</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -7083,7 +7083,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D270" t="n">
@@ -7108,7 +7108,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D271" t="n">
@@ -7483,7 +7483,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D286" t="n">
@@ -7508,7 +7508,7 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D287" t="n">
@@ -7998,23 +7998,148 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
+          <t>23:09:10</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>23:29</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D307" t="n">
+        <v>20</v>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
           <t>21:33:35</t>
         </is>
       </c>
-      <c r="B307" t="inlineStr">
+      <c r="B308" t="inlineStr">
         <is>
           <t>23:30</t>
         </is>
       </c>
-      <c r="C307" t="inlineStr">
+      <c r="C308" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D307" t="n">
+      <c r="D308" t="n">
         <v>117</v>
       </c>
-      <c r="E307" t="inlineStr">
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>23:09:10</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>23:34</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D309" t="n">
+        <v>25</v>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>23:09:10</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>23:41</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D310" t="n">
+        <v>32</v>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>23:09:10</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>23:50</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D311" t="n">
+        <v>41</v>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>23:09:10</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>23:54</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D312" t="n">
+        <v>45</v>
+      </c>
+      <c r="E312" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8031,7 +8156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8044,14 +8169,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 21:33:35</t>
+          <t>Última actualización: 23:09:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 50</t>
+          <t>Total filas: 52</t>
         </is>
       </c>
     </row>
@@ -8220,7 +8345,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -8245,7 +8370,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -9310,23 +9435,73 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
+          <t>23:09:10</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>23:29</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>20</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>21:33:35</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>23:30</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D55" t="n">
+      <c r="D56" t="n">
         <v>117</v>
       </c>
-      <c r="E55" t="inlineStr">
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>23:09:10</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>23:41</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>32</v>
+      </c>
+      <c r="E57" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9356,7 +9531,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 21:33:35</t>
+          <t>Última actualización: 23:09:10</t>
         </is>
       </c>
     </row>

</xml_diff>